<commit_message>
Job sweep: add India rows 146-150, applied-company reminders, audit-clean workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DTEXuchYd8TgLUXdwKuKDn
</commit_message>
<xml_diff>
--- a/job_sweep/Best_Fit_Jobs_By_Deadline.xlsx
+++ b/job_sweep/Best_Fit_Jobs_By_Deadline.xlsx
@@ -14,9 +14,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Apply By Deadline'!$A$1:$V$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Apply By Deadline'!$A$1:$V$64</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Opening Soon'!$A$1:$F$27</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Closed - Excluded'!$A$1:$E$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Closed - Excluded'!$A$1:$E$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Coverage'!$A$1:$H$260</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V59"/>
+  <dimension ref="A1:V64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2712,32 +2712,32 @@
       <c r="C23" s="12" t="n"/>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Simon-Kucher</t>
+          <t>Razorpay</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Life Sciences Consulting Internship (autumn/winter start dates) - London</t>
+          <t>Associate Business Analyst (Off Campus 2026)</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Consulting</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Nov 2026 / winter 2026–27</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
@@ -2750,12 +2750,12 @@
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>Graduate-level pricing/strategy consulting internship that feeds full-time consultant hiring; MCC costing + Excel modelling</t>
+          <t>Fresher BA at India's leading payments fintech; SQL/Python/Power BI + FinTech MSc + BA case study</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>Graduates (internships aimed at those who have already graduated)</t>
+          <t>Bachelor's/Master's, any batch</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
@@ -2765,7 +2765,7 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>N/A (India)</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
@@ -2775,23 +2775,23 @@
       </c>
       <c r="Q23" s="5" t="inlineStr">
         <is>
-          <t>https://targetjobs.co.uk/jobs/life-sciences-internship-autumn-winter-start-dates-185724</t>
+          <t>https://www.fresheroffcampus.com/razorpay-off-campus-hiring-fresher/</t>
         </is>
       </c>
       <c r="R23" s="2" t="inlineStr">
         <is>
-          <t>TargetJobs / managementconsulted (via web search)</t>
+          <t>FresherOffCampus (via web search)</t>
         </is>
       </c>
       <c r="S23" s="2" t="inlineStr">
         <is>
-          <t>No deadline in snippet</t>
+          <t>No deadline shown</t>
         </is>
       </c>
       <c r="T23" s="2" t="inlineStr"/>
       <c r="U23" s="2" t="inlineStr">
         <is>
-          <t>INTERNSHIP (graduate). Life-sciences sector focus. Apply ASAP — Nov 2026 start.</t>
+          <t>Aggregator listing — verify on Razorpay careers. Apply ASAP — may close early.</t>
         </is>
       </c>
       <c r="V23" s="6" t="n">
@@ -2810,7 +2810,7 @@
       <c r="C24" s="12" t="n"/>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Elixirr</t>
+          <t>Simon-Kucher</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -2820,7 +2820,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2027 Graduate Analyst (Consulting Analyst)</t>
+          <t>Life Sciences Consulting Internship (autumn/winter start dates) - London</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -2830,12 +2830,12 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>London (City HQ)</t>
+          <t>London</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Summer 2027</t>
+          <t>Nov 2026 / winter 2026–27</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -2848,12 +2848,12 @@
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>Challenger consultancy grad analyst; Excel/PowerPoint, quant + qual analysis from MCC and BA case study</t>
+          <t>Graduate-level pricing/strategy consulting internship that feeds full-time consultant hiring; MCC costing + Excel modelling</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>2027 graduate, any discipline; Excel &amp; PowerPoint</t>
+          <t>Graduates (internships aimed at those who have already graduated)</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
@@ -2863,7 +2863,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>Must be UK work-authorised without current or future sponsorship</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
@@ -2873,23 +2873,23 @@
       </c>
       <c r="Q24" s="5" t="inlineStr">
         <is>
-          <t>https://targetjobs.co.uk/jobs/2027-graduate-analyst-246849</t>
+          <t>https://targetjobs.co.uk/jobs/life-sciences-internship-autumn-winter-start-dates-185724</t>
         </is>
       </c>
       <c r="R24" s="2" t="inlineStr">
         <is>
-          <t>TargetJobs / Elixirr site (via web search)</t>
+          <t>TargetJobs / managementconsulted (via web search)</t>
         </is>
       </c>
       <c r="S24" s="2" t="inlineStr">
         <is>
-          <t>No deadline shown</t>
+          <t>No deadline in snippet</t>
         </is>
       </c>
       <c r="T24" s="2" t="inlineStr"/>
       <c r="U24" s="2" t="inlineStr">
         <is>
-          <t>2027 START. Eligibility risk: asks for 2027 graduates and no future sponsorship — confirm they'd accept a 2026 MSc graduate.</t>
+          <t>INTERNSHIP (graduate). Life-sciences sector focus. Apply ASAP — Nov 2026 start.</t>
         </is>
       </c>
       <c r="V24" s="6" t="n">
@@ -2908,7 +2908,7 @@
       <c r="C25" s="12" t="n"/>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Newton Europe</t>
+          <t>Elixirr</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -2918,7 +2918,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Graduate Consultant</t>
+          <t>2027 Graduate Analyst (Consulting Analyst)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -2928,30 +2928,30 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>UK (Oxfordshire HQ; client-site travel)</t>
+          <t>London (City HQ)</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Summer 2027</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>£48,000 + £2,500 joining bonus</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="K25" s="2" t="n">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>Operations-improvement consulting grad role; MCC operating-cost model and root-cause analysis map directly</t>
+          <t>Challenger consultancy grad analyst; Excel/PowerPoint, quant + qual analysis from MCC and BA case study</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>Any degree</t>
+          <t>2027 graduate, any discipline; Excel &amp; PowerPoint</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
@@ -2961,7 +2961,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Must be UK work-authorised without current or future sponsorship</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
@@ -2971,23 +2971,23 @@
       </c>
       <c r="Q25" s="5" t="inlineStr">
         <is>
-          <t>https://www.brightnetwork.co.uk/graduate-jobs/newton-europe/graduate-consultant-3</t>
+          <t>https://targetjobs.co.uk/jobs/2027-graduate-analyst-246849</t>
         </is>
       </c>
       <c r="R25" s="2" t="inlineStr">
         <is>
-          <t>Bright Network / Sanctuary Graduates (via web search)</t>
+          <t>TargetJobs / Elixirr site (via web search)</t>
         </is>
       </c>
       <c r="S25" s="2" t="inlineStr">
         <is>
-          <t>Application deadline rolling — apply as soon as possible</t>
+          <t>No deadline shown</t>
         </is>
       </c>
       <c r="T25" s="2" t="inlineStr"/>
       <c r="U25" s="2" t="inlineStr">
         <is>
-          <t>Apply ASAP — may close early. Listing may refer to an earlier intake; verify on company site.</t>
+          <t>2027 START. Eligibility risk: asks for 2027 graduates and no future sponsorship — confirm they'd accept a 2026 MSc graduate.</t>
         </is>
       </c>
       <c r="V25" s="6" t="n">
@@ -3006,7 +3006,7 @@
       <c r="C26" s="12" t="n"/>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Turner &amp; Townsend</t>
+          <t>Newton Europe</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -3016,7 +3016,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Graduate Programme 2027 - Project Management and Project Controls</t>
+          <t>Graduate Consultant</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -3026,17 +3026,17 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>UK (multiple offices)</t>
+          <t>UK (Oxfordshire HQ; client-site travel)</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>£48,000 + £2,500 joining bonus</t>
         </is>
       </c>
       <c r="K26" s="2" t="n">
@@ -3044,12 +3044,12 @@
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>Project controls = cost/schedule analytics; your £50M facility costing and operating-cost model fit</t>
+          <t>Operations-improvement consulting grad role; MCC operating-cost model and root-cause analysis map directly</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Any degree</t>
         </is>
       </c>
       <c r="N26" s="2" t="inlineStr">
@@ -3069,23 +3069,23 @@
       </c>
       <c r="Q26" s="5" t="inlineStr">
         <is>
-          <t>https://www.gradcracker.com/hub/686/turner-and-townsend/graduate-job/83125/graduate-programme-2027-project-management-and-project-controls</t>
+          <t>https://www.brightnetwork.co.uk/graduate-jobs/newton-europe/graduate-consultant-3</t>
         </is>
       </c>
       <c r="R26" s="2" t="inlineStr">
         <is>
-          <t>Gradcracker (via web search)</t>
+          <t>Bright Network / Sanctuary Graduates (via web search)</t>
         </is>
       </c>
       <c r="S26" s="2" t="inlineStr">
         <is>
-          <t>No closing date shown</t>
+          <t>Application deadline rolling — apply as soon as possible</t>
         </is>
       </c>
       <c r="T26" s="2" t="inlineStr"/>
       <c r="U26" s="2" t="inlineStr">
         <is>
-          <t>2027 START.</t>
+          <t>Apply ASAP — may close early. Listing may refer to an earlier intake; verify on company site.</t>
         </is>
       </c>
       <c r="V26" s="6" t="n">
@@ -3104,7 +3104,7 @@
       <c r="C27" s="12" t="n"/>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Mott MacDonald</t>
+          <t>Turner &amp; Townsend</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2027 UK Graduate Management Consultancy Career Path</t>
+          <t>Graduate Programme 2027 - Project Management and Project Controls</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -3124,7 +3124,7 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>UK (multiple offices)</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
@@ -3142,12 +3142,12 @@
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>Business cases, resilience and digital operations consulting; MCC business case + BA case study</t>
+          <t>Project controls = cost/schedule analytics; your £50M facility costing and operating-cost model fit</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>Business/Economics/Maths/Analytics background; &lt;12 months experience; degree 2025+</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr">
@@ -3167,7 +3167,7 @@
       </c>
       <c r="Q27" s="5" t="inlineStr">
         <is>
-          <t>https://www.gradcracker.com/hub/3/mott-macdonald/graduate-job/84119/2027-uk-graduate-management-consultancy-career-path</t>
+          <t>https://www.gradcracker.com/hub/686/turner-and-townsend/graduate-job/83125/graduate-programme-2027-project-management-and-project-controls</t>
         </is>
       </c>
       <c r="R27" s="2" t="inlineStr">
@@ -3183,7 +3183,7 @@
       <c r="T27" s="2" t="inlineStr"/>
       <c r="U27" s="2" t="inlineStr">
         <is>
-          <t>2027 START. Sister roles close mid-Oct — apply now.</t>
+          <t>2027 START.</t>
         </is>
       </c>
       <c r="V27" s="6" t="n">
@@ -3202,7 +3202,7 @@
       <c r="C28" s="12" t="n"/>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>BDO UK</t>
+          <t>Mott MacDonald</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -3212,7 +3212,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2027 Advisory Graduate Programme - Midlands</t>
+          <t>2027 UK Graduate Management Consultancy Career Path</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -3222,17 +3222,17 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Midlands (Birmingham)</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>20 Sep 2027</t>
+          <t>2027</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>£33,000 (London AM listing; Midlands not stated)</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="K28" s="2" t="n">
@@ -3240,17 +3240,17 @@
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>Advisory grad in Birmingham (restructuring, forensics, M&amp;A); Excel modelling + analytics tag</t>
+          <t>Business cases, resilience and digital operations consulting; MCC business case + BA case study</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>2:2 and above</t>
+          <t>Business/Economics/Maths/Analytics background; &lt;12 months experience; degree 2025+</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>Online application → online assessments → video interview → virtual AC → final in-person interview</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="O28" s="2" t="inlineStr">
@@ -3265,23 +3265,23 @@
       </c>
       <c r="Q28" s="5" t="inlineStr">
         <is>
-          <t>https://targetjobs.co.uk/jobs/2027-advisory-graduate-programme-midlands-245531</t>
+          <t>https://www.gradcracker.com/hub/3/mott-macdonald/graduate-job/84119/2027-uk-graduate-management-consultancy-career-path</t>
         </is>
       </c>
       <c r="R28" s="2" t="inlineStr">
         <is>
-          <t>TargetJobs (via web search)</t>
+          <t>Gradcracker (via web search)</t>
         </is>
       </c>
       <c r="S28" s="2" t="inlineStr">
         <is>
-          <t>Midlands date not shown; Scotland and NE&amp;W listings close 15 Nov 2026</t>
+          <t>No closing date shown</t>
         </is>
       </c>
       <c r="T28" s="2" t="inlineStr"/>
       <c r="U28" s="2" t="inlineStr">
         <is>
-          <t>2027 START. Birmingham bonus. Check Midlands closing date.</t>
+          <t>2027 START. Sister roles close mid-Oct — apply now.</t>
         </is>
       </c>
       <c r="V28" s="6" t="n">
@@ -3300,7 +3300,7 @@
       <c r="C29" s="12" t="n"/>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>KPMG (UK)</t>
+          <t>BDO UK</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -3310,7 +3310,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>KPMG 2027 Technology Consulting in Tax Graduate Programme - London</t>
+          <t>2027 Advisory Graduate Programme - Midlands</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -3320,50 +3320,50 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Midlands (Birmingham)</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>Autumn 2027</t>
+          <t>20 Sep 2027</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>£33,000 (London AM listing; Midlands not stated)</t>
         </is>
       </c>
       <c r="K29" s="2" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>Graduate tech-consulting track distinct from your Consulting application; CS degree + BA documentation skills fit</t>
+          <t>Advisory grad in Birmingham (restructuring, forensics, M&amp;A); Excel modelling + analytics tag</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>See KPMG careers portal entry requirements</t>
+          <t>2:2 and above</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Online application → online assessments → video interview → virtual AC → final in-person interview</t>
         </is>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>Limited sponsorship for London consulting/technology programmes (offer acceptance by 1 June 2027)</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="Q29" s="5" t="inlineStr">
         <is>
-          <t>https://targetjobs.co.uk/jobs/kpmg-2027-technology-consulting-tax-graduate-programme-london-243587</t>
+          <t>https://targetjobs.co.uk/jobs/2027-advisory-graduate-programme-midlands-245531</t>
         </is>
       </c>
       <c r="R29" s="2" t="inlineStr">
@@ -3373,13 +3373,13 @@
       </c>
       <c r="S29" s="2" t="inlineStr">
         <is>
-          <t>Deadline vacancy-specific</t>
+          <t>Midlands date not shown; Scotland and NE&amp;W listings close 15 Nov 2026</t>
         </is>
       </c>
       <c r="T29" s="2" t="inlineStr"/>
       <c r="U29" s="2" t="inlineStr">
         <is>
-          <t>2027 START. Apply ASAP — may close early. Verify on company site.</t>
+          <t>2027 START. Birmingham bonus. Check Midlands closing date.</t>
         </is>
       </c>
       <c r="V29" s="6" t="n">
@@ -3398,7 +3398,7 @@
       <c r="C30" s="12" t="n"/>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Accenture (UK)</t>
+          <t>KPMG (UK)</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -3408,22 +3408,22 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>London Technology Analyst Graduate Programme 2027 - 2028</t>
+          <t>KPMG 2027 Technology Consulting in Tax Graduate Programme - London</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Graduate Programme</t>
+          <t>Consulting</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>London (also Birmingham listing)</t>
+          <t>London</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>Sep 2027 – Aug 2028</t>
+          <t>Autumn 2027</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -3436,22 +3436,22 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>First roles typically Data Analyst / Business Analyst; your BA case study and SQL/Power BI fit directly</t>
+          <t>Graduate tech-consulting track distinct from your Consulting application; CS degree + BA documentation skills fit</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>No coding skills needed; analytical thinking, curious/growth mindset; 3 days/week in office</t>
+          <t>See KPMG careers portal entry requirements</t>
         </is>
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>Interviews typically Nov–Spring; no technical assessments</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Limited sponsorship for London consulting/technology programmes (offer acceptance by 1 June 2027)</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
@@ -3461,23 +3461,23 @@
       </c>
       <c r="Q30" s="5" t="inlineStr">
         <is>
-          <t>https://www.gradcracker.com/hub/269/accenture/graduate-job/85118/london-technology-analyst-graduate-programme-2027-2028</t>
+          <t>https://targetjobs.co.uk/jobs/kpmg-2027-technology-consulting-tax-graduate-programme-london-243587</t>
         </is>
       </c>
       <c r="R30" s="2" t="inlineStr">
         <is>
-          <t>Gradcracker / TargetJobs (via web search)</t>
+          <t>TargetJobs (via web search)</t>
         </is>
       </c>
       <c r="S30" s="2" t="inlineStr">
         <is>
-          <t>Accenture doesn't post deadlines; closes once enough applications</t>
+          <t>Deadline vacancy-specific</t>
         </is>
       </c>
       <c r="T30" s="2" t="inlineStr"/>
       <c r="U30" s="2" t="inlineStr">
         <is>
-          <t>2027 START. Apply ASAP — may close early. Birmingham version: gradcracker.com/hub/269/accenture/graduate-job/85121</t>
+          <t>2027 START. Apply ASAP — may close early. Verify on company site.</t>
         </is>
       </c>
       <c r="V30" s="6" t="n">
@@ -3496,7 +3496,7 @@
       <c r="C31" s="12" t="n"/>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>LSEG (London Stock Exchange Group)</t>
+          <t>Accenture (UK)</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -3506,7 +3506,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Business Graduate Programme (Data and Analytics)</t>
+          <t>London Technology Analyst Graduate Programme 2027 - 2028</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -3516,12 +3516,12 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>London (also Birmingham listing)</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>Sep 2027</t>
+          <t>Sep 2027 – Aug 2028</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
@@ -3534,17 +3534,17 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>Data &amp; Analytics division grad track (Analytics or Data &amp; Feeds); your FinBERT/Power BI dissertation and FinTech MSc fit</t>
+          <t>First roles typically Data Analyst / Business Analyst; your BA case study and SQL/Power BI fit directly</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>Completed studies in 2026, or finishing before summer 2027</t>
+          <t>No coding skills needed; analytical thinking, curious/growth mindset; 3 days/week in office</t>
         </is>
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Interviews typically Nov–Spring; no technical assessments</t>
         </is>
       </c>
       <c r="O31" s="2" t="inlineStr">
@@ -3559,23 +3559,23 @@
       </c>
       <c r="Q31" s="5" t="inlineStr">
         <is>
-          <t>https://www.gradcracker.com/hub/300/london-stock-exchange-group/graduate-job/84076/business-graduate-programmedata-and-analytics</t>
+          <t>https://www.gradcracker.com/hub/269/accenture/graduate-job/85118/london-technology-analyst-graduate-programme-2027-2028</t>
         </is>
       </c>
       <c r="R31" s="2" t="inlineStr">
         <is>
-          <t>eFinancialCareers (via web search)</t>
+          <t>Gradcracker / TargetJobs (via web search)</t>
         </is>
       </c>
       <c r="S31" s="2" t="inlineStr">
         <is>
-          <t>eFinancialCareers: 'application close 28 November' (year cut off in snippet)</t>
+          <t>Accenture doesn't post deadlines; closes once enough applications</t>
         </is>
       </c>
       <c r="T31" s="2" t="inlineStr"/>
       <c r="U31" s="2" t="inlineStr">
         <is>
-          <t>2027 START. Likely 28 Nov 2026 but year not visible — treat as rolling and apply early.</t>
+          <t>2027 START. Apply ASAP — may close early. Birmingham version: gradcracker.com/hub/269/accenture/graduate-job/85121</t>
         </is>
       </c>
       <c r="V31" s="6" t="n">
@@ -3604,7 +3604,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst Graduate Programme</t>
+          <t>Business Graduate Programme (Data and Analytics)</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -3632,12 +3632,12 @@
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>Graduate BA programme with Markets division rotation; BA case study + FinTech MSc fit</t>
+          <t>Data &amp; Analytics division grad track (Analytics or Data &amp; Feeds); your FinBERT/Power BI dissertation and FinTech MSc fit</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Completed studies in 2026, or finishing before summer 2027</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr">
@@ -3657,23 +3657,23 @@
       </c>
       <c r="Q32" s="5" t="inlineStr">
         <is>
-          <t>https://targetjobs.co.uk/jobs/business-analyst-graduate-programme-242317</t>
+          <t>https://www.gradcracker.com/hub/300/london-stock-exchange-group/graduate-job/84076/business-graduate-programmedata-and-analytics</t>
         </is>
       </c>
       <c r="R32" s="2" t="inlineStr">
         <is>
-          <t>TargetJobs / Built In London (via web search)</t>
+          <t>eFinancialCareers (via web search)</t>
         </is>
       </c>
       <c r="S32" s="2" t="inlineStr">
         <is>
-          <t>No closing date shown</t>
+          <t>eFinancialCareers: 'application close 28 November' (year cut off in snippet)</t>
         </is>
       </c>
       <c r="T32" s="2" t="inlineStr"/>
       <c r="U32" s="2" t="inlineStr">
         <is>
-          <t>2027 START. Sister programme closes 20 Oct — apply ASAP.</t>
+          <t>2027 START. Likely 28 Nov 2026 but year not visible — treat as rolling and apply early.</t>
         </is>
       </c>
       <c r="V32" s="6" t="n">
@@ -3692,7 +3692,7 @@
       <c r="C33" s="12" t="n"/>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Checkout.com</t>
+          <t>LSEG (London Stock Exchange Group)</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -3702,22 +3702,22 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Data Analytics Graduate (#NextGen Graduate Program)</t>
+          <t>Business Analyst Graduate Programme</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Graduate Programme</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>London (HQ; location not explicit in excerpt)</t>
+          <t>London</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Sep 2027</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
@@ -3730,12 +3730,12 @@
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>Payments fintech grad data role open to those graduated within 2 years; SQL/Python/Power BI + FinTech MSc</t>
+          <t>Graduate BA programme with Markets division rotation; BA case study + FinTech MSc fit</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>Graduated by July 2026 or within last 2 years; quantitative degree</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="N33" s="2" t="inlineStr">
@@ -3750,28 +3750,28 @@
       </c>
       <c r="P33" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="Q33" s="5" t="inlineStr">
         <is>
-          <t>https://targetjobs.co.uk/jobs/data-analytics-graduate-214568</t>
+          <t>https://targetjobs.co.uk/jobs/business-analyst-graduate-programme-242317</t>
         </is>
       </c>
       <c r="R33" s="2" t="inlineStr">
         <is>
-          <t>TargetJobs (via web search)</t>
+          <t>TargetJobs / Built In London (via web search)</t>
         </is>
       </c>
       <c r="S33" s="2" t="inlineStr">
         <is>
-          <t>No deadline in excerpt</t>
+          <t>No closing date shown</t>
         </is>
       </c>
       <c r="T33" s="2" t="inlineStr"/>
       <c r="U33" s="2" t="inlineStr">
         <is>
-          <t>Listing may be from the 2026 cycle — check it is still open. Verify location.</t>
+          <t>2027 START. Sister programme closes 20 Oct — apply ASAP.</t>
         </is>
       </c>
       <c r="V33" s="6" t="n">
@@ -3790,7 +3790,7 @@
       <c r="C34" s="12" t="n"/>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>SumUp</t>
+          <t>Checkout.com</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -3800,7 +3800,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst (Consumer Bank)</t>
+          <t>Data Analytics Graduate (#NextGen Graduate Program)</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -3810,7 +3810,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>London (in office)</t>
+          <t>London (HQ; location not explicit in excerpt)</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -3828,12 +3828,12 @@
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>Entry-level fintech data analyst — KPI reporting and A/B testing; your Power BI/KPI and Python stats work fit</t>
+          <t>Payments fintech grad data role open to those graduated within 2 years; SQL/Python/Power BI + FinTech MSc</t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>KPI reporting, A/B testing support, data modelling collaboration</t>
+          <t>Graduated by July 2026 or within last 2 years; quantitative degree</t>
         </is>
       </c>
       <c r="N34" s="2" t="inlineStr">
@@ -3853,23 +3853,23 @@
       </c>
       <c r="Q34" s="5" t="inlineStr">
         <is>
-          <t>https://builtinlondon.uk/job/data-analyst/9450609</t>
+          <t>https://targetjobs.co.uk/jobs/data-analytics-graduate-214568</t>
         </is>
       </c>
       <c r="R34" s="2" t="inlineStr">
         <is>
-          <t>Built In London (via web search)</t>
+          <t>TargetJobs (via web search)</t>
         </is>
       </c>
       <c r="S34" s="2" t="inlineStr">
         <is>
-          <t>No deadline shown</t>
+          <t>No deadline in excerpt</t>
         </is>
       </c>
       <c r="T34" s="2" t="inlineStr"/>
       <c r="U34" s="2" t="inlineStr">
         <is>
-          <t>Apply ASAP — may close early. Verify still live on SumUp careers.</t>
+          <t>Listing may be from the 2026 cycle — check it is still open. Verify location.</t>
         </is>
       </c>
       <c r="V34" s="6" t="n">
@@ -3888,7 +3888,7 @@
       <c r="C35" s="12" t="n"/>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Zopa</t>
+          <t>SumUp</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -3898,27 +3898,27 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2027 Graduate Analyst</t>
+          <t>Data Analyst (Consumer Bank)</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Graduate Programme</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>London (hybrid)</t>
+          <t>London (in office)</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>Not stated (2026 cohort: £42k)</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="K35" s="2" t="n">
@@ -3926,17 +3926,17 @@
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>Rotational analytics grad scheme at a digital bank (credit strategy, product analytics, data science, risk); dissertation NLP/econometrics + FinTech MSc</t>
+          <t>Entry-level fintech data analyst — KPI reporting and A/B testing; your Power BI/KPI and Python stats work fit</t>
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>KPI reporting, A/B testing support, data modelling collaboration</t>
         </is>
       </c>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>4-month structured training, 4 placements with a project each</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="O35" s="2" t="inlineStr">
@@ -3951,23 +3951,23 @@
       </c>
       <c r="Q35" s="5" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/zopa/962f3756-6e45-480f-984c-64e024b57c4f</t>
+          <t>https://builtinlondon.uk/job/data-analyst/9450609</t>
         </is>
       </c>
       <c r="R35" s="2" t="inlineStr">
         <is>
-          <t>Company site (Lever) via web search</t>
+          <t>Built In London (via web search)</t>
         </is>
       </c>
       <c r="S35" s="2" t="inlineStr">
         <is>
-          <t>No deadline shown; posted recently</t>
+          <t>No deadline shown</t>
         </is>
       </c>
       <c r="T35" s="2" t="inlineStr"/>
       <c r="U35" s="2" t="inlineStr">
         <is>
-          <t>2027 START. Apply ASAP — may close early.</t>
+          <t>Apply ASAP — may close early. Verify still live on SumUp careers.</t>
         </is>
       </c>
       <c r="V35" s="6" t="n">
@@ -3986,7 +3986,7 @@
       <c r="C36" s="12" t="n"/>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Stroud International</t>
+          <t>Zopa</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -3996,27 +3996,27 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Associate Consultant (London)</t>
+          <t>2027 Graduate Analyst</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Consulting</t>
+          <t>Graduate Programme</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>London (hybrid)</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>2027</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Not stated (2026 cohort: £42k)</t>
         </is>
       </c>
       <c r="K36" s="2" t="n">
@@ -4024,17 +4024,17 @@
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>Entry operations-consulting role working alongside clients; root-cause analysis and MCC operating model work transfer</t>
+          <t>Rotational analytics grad scheme at a digital bank (credit strategy, product analytics, data science, risk); dissertation NLP/econometrics + FinTech MSc</t>
         </is>
       </c>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>Must attend an information session after applying</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>Apply → attend information session → interviews</t>
+          <t>4-month structured training, 4 placements with a project each</t>
         </is>
       </c>
       <c r="O36" s="2" t="inlineStr">
@@ -4049,23 +4049,23 @@
       </c>
       <c r="Q36" s="5" t="inlineStr">
         <is>
-          <t>https://stroudinternational-1690276198.teamtailor.com/jobs/6938267-associate-consultant-london</t>
+          <t>https://jobs.lever.co/zopa/962f3756-6e45-480f-984c-64e024b57c4f</t>
         </is>
       </c>
       <c r="R36" s="2" t="inlineStr">
         <is>
-          <t>Company site (Teamtailor) via web search</t>
+          <t>Company site (Lever) via web search</t>
         </is>
       </c>
       <c r="S36" s="2" t="inlineStr">
         <is>
-          <t>Undated posting; no deadline</t>
+          <t>No deadline shown; posted recently</t>
         </is>
       </c>
       <c r="T36" s="2" t="inlineStr"/>
       <c r="U36" s="2" t="inlineStr">
         <is>
-          <t>Apply ASAP — may close early. Check london-office-recruitment page for session dates.</t>
+          <t>2027 START. Apply ASAP — may close early.</t>
         </is>
       </c>
       <c r="V36" s="6" t="n">
@@ -4084,50 +4084,50 @@
       <c r="C37" s="12" t="n"/>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Barclays (UK)</t>
+          <t>Razorpay</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2027 Operations Analyst Graduate Programme</t>
+          <t>Analyst, Business Operations</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Graduate Programme</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>UK (multiple listings)</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>Aug 2027</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Not stated (aggregator estimate ₹6–8 LPA)</t>
         </is>
       </c>
       <c r="K37" s="2" t="n">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>2-yr Explorer programme, three 8-month rotations in banking operations; process/root-cause analysis and BPMN work fit</t>
+          <t>Entry ops-analyst role for 2024–2026 batches; process analysis and stakeholder coordination</t>
         </is>
       </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>2024, 2025 or 2026 batch graduates</t>
         </is>
       </c>
       <c r="N37" s="2" t="inlineStr">
@@ -4137,33 +4137,33 @@
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>Accepts applicants who need visa sponsorship</t>
+          <t>N/A (India)</t>
         </is>
       </c>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="Q37" s="5" t="inlineStr">
         <is>
-          <t>https://www.gradcracker.com/hub/180/barclays/graduate-job/85643/2027-operations-analyst-graduate-programme</t>
+          <t>https://fresherjobinfo.in/?p=40214</t>
         </is>
       </c>
       <c r="R37" s="2" t="inlineStr">
         <is>
-          <t>Gradcracker (via web search)</t>
+          <t>FresherJobInfo (via web search)</t>
         </is>
       </c>
       <c r="S37" s="2" t="inlineStr">
         <is>
-          <t>May close early due to application volumes — apply early</t>
+          <t>No deadline shown</t>
         </is>
       </c>
       <c r="T37" s="2" t="inlineStr"/>
       <c r="U37" s="2" t="inlineStr">
         <is>
-          <t>2027 START. Apply ASAP — may close early. Verify on company site.</t>
+          <t>Description reads like payroll-product customer onboarding. Verify on Razorpay careers.</t>
         </is>
       </c>
       <c r="V37" s="6" t="n">
@@ -4182,32 +4182,32 @@
       <c r="C38" s="12" t="n"/>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>RSM UK</t>
+          <t>India SaaS (Freshworks, Zoho, Postman, Chargebee, BrowserStack, InMobi, Delhivery, PolicyBazaar, Navi, Angel One)</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Consulting Graduate - Bristol - September 2027</t>
+          <t>BrowserStack — Business Analyst Intern (Mumbai)</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Consulting</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Bristol</t>
+          <t>Mumbai</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>Sep 2027</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -4216,16 +4216,16 @@
         </is>
       </c>
       <c r="K38" s="2" t="n">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>Consulting grad (Risk Assurance / Finance Function Support); MCC consulting + root-cause analysis</t>
+          <t>BA internship open to 2025–2027 graduates; SQL, advanced Excel and Python match</t>
         </is>
       </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>Honours degree (predicted/obtained); permanent UK right to work; travel to client sites</t>
+          <t>Graduation year 2025, 2026 or 2027; strong SQL, advanced Excel, some Python/R</t>
         </is>
       </c>
       <c r="N38" s="2" t="inlineStr">
@@ -4235,7 +4235,7 @@
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>Permanent right to work required</t>
+          <t>N/A (India)</t>
         </is>
       </c>
       <c r="P38" s="2" t="inlineStr">
@@ -4245,12 +4245,12 @@
       </c>
       <c r="Q38" s="5" t="inlineStr">
         <is>
-          <t>https://targetjobs.co.uk/jobs/consulting-graduate-bristol-september-2027-239989</t>
+          <t>https://myinternships.in/job/browserstack-business-analyst-intern-mumbai-b6582b</t>
         </is>
       </c>
       <c r="R38" s="2" t="inlineStr">
         <is>
-          <t>TargetJobs (via web search)</t>
+          <t>MyInternships (via web search)</t>
         </is>
       </c>
       <c r="S38" s="2" t="inlineStr">
@@ -4261,7 +4261,7 @@
       <c r="T38" s="2" t="inlineStr"/>
       <c r="U38" s="2" t="inlineStr">
         <is>
-          <t>2027 START. Check RSM site for a London/Birmingham consulting variant. Eligibility risk on 'permanent right to work'.</t>
+          <t>INTERNSHIP (open to recent graduates). Status unclear — verify on BrowserStack careers.</t>
         </is>
       </c>
       <c r="V38" s="6" t="n">
@@ -4280,7 +4280,7 @@
       <c r="C39" s="12" t="n"/>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Wise</t>
+          <t>Stroud International</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -4290,12 +4290,12 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Graduate Analyst - London</t>
+          <t>Associate Consultant (London)</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Consulting</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -4314,21 +4314,21 @@
         </is>
       </c>
       <c r="K39" s="2" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>Graduate analytics role at a fintech; SQL/Python/Power BI dashboarding from your dissertation and ESG dashboard project fit</t>
+          <t>Entry operations-consulting role working alongside clients; root-cause analysis and MCC operating model work transfer</t>
         </is>
       </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>2025/2026 graduate (Bachelor's/Master's) in data/CS/STEM/economics (per related Wise grad listing)</t>
+          <t>Must attend an information session after applying</t>
         </is>
       </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Apply → attend information session → interviews</t>
         </is>
       </c>
       <c r="O39" s="2" t="inlineStr">
@@ -4338,28 +4338,28 @@
       </c>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="Q39" s="5" t="inlineStr">
         <is>
-          <t>https://wise.jobs/job/graduate-analyst-london-in-london-jid-3837</t>
+          <t>https://stroudinternational-1690276198.teamtailor.com/jobs/6938267-associate-consultant-london</t>
         </is>
       </c>
       <c r="R39" s="2" t="inlineStr">
         <is>
-          <t>Web search (wise.jobs / TargetJobs)</t>
+          <t>Company site (Teamtailor) via web search</t>
         </is>
       </c>
       <c r="S39" s="2" t="inlineStr">
         <is>
-          <t>No deadline shown; one Wise grad analyst listing marked 'This vacancy has now expired'</t>
+          <t>Undated posting; no deadline</t>
         </is>
       </c>
       <c r="T39" s="2" t="inlineStr"/>
       <c r="U39" s="2" t="inlineStr">
         <is>
-          <t>Status uncertain — a sister listing has expired; check it is still open. Apply ASAP — may close early.</t>
+          <t>Apply ASAP — may close early. Check london-office-recruitment page for session dates.</t>
         </is>
       </c>
       <c r="V39" s="6" t="n">
@@ -4378,7 +4378,7 @@
       <c r="C40" s="12" t="n"/>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Ebury</t>
+          <t>Barclays (UK)</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -4388,22 +4388,22 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Graduate Banking Operations Analyst</t>
+          <t>2027 Operations Analyst Graduate Programme</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Graduate Programme</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>London (hybrid, 4 days office)</t>
+          <t>UK (multiple listings)</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Aug 2027</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -4412,11 +4412,11 @@
         </is>
       </c>
       <c r="K40" s="2" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>Graduate operations analyst at an FX/payments fintech; process documentation and stakeholder coordination from your BA case study</t>
+          <t>2-yr Explorer programme, three 8-month rotations in banking operations; process/root-cause analysis and BPMN work fit</t>
         </is>
       </c>
       <c r="M40" s="2" t="inlineStr">
@@ -4431,33 +4431,33 @@
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Accepts applicants who need visa sponsorship</t>
         </is>
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="Q40" s="5" t="inlineStr">
         <is>
-          <t>https://targetjobs.co.uk/jobs/graduate-banking-operations-analyst-213626</t>
+          <t>https://www.gradcracker.com/hub/180/barclays/graduate-job/85643/2027-operations-analyst-graduate-programme</t>
         </is>
       </c>
       <c r="R40" s="2" t="inlineStr">
         <is>
-          <t>TargetJobs (via web search)</t>
+          <t>Gradcracker (via web search)</t>
         </is>
       </c>
       <c r="S40" s="2" t="inlineStr">
         <is>
-          <t>No deadline shown</t>
+          <t>May close early due to application volumes — apply early</t>
         </is>
       </c>
       <c r="T40" s="2" t="inlineStr"/>
       <c r="U40" s="2" t="inlineStr">
         <is>
-          <t>Listing may be from an earlier cycle — check it is still open. Role is operational (account opening, mandates).</t>
+          <t>2027 START. Apply ASAP — may close early. Verify on company site.</t>
         </is>
       </c>
       <c r="V40" s="6" t="n">
@@ -4476,7 +4476,7 @@
       <c r="C41" s="12" t="n"/>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Funding Circle</t>
+          <t>RSM UK</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -4486,40 +4486,40 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst (London, hybrid)</t>
+          <t>Consulting Graduate - Bristol - September 2027</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Consulting</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>London (hybrid, 3 days office)</t>
+          <t>Bristol</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Sep 2027</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>Not stated (Home Office going rate listed as £34,900)</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="K41" s="2" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>SME-lending fintech data role open to recent grads with strong data skills; SQL/Tableau/Python + CS degree</t>
+          <t>Consulting grad (Risk Assurance / Finance Function Support); MCC consulting + root-cause analysis</t>
         </is>
       </c>
       <c r="M41" s="2" t="inlineStr">
         <is>
-          <t>Numerical/data degree; 1–2 yrs OR recent graduate with strong data skills; SQL, Tableau</t>
+          <t>Honours degree (predicted/obtained); permanent UK right to work; travel to client sites</t>
         </is>
       </c>
       <c r="N41" s="2" t="inlineStr">
@@ -4529,7 +4529,7 @@
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>Employer holds sponsor licence (listing)</t>
+          <t>Permanent right to work required</t>
         </is>
       </c>
       <c r="P41" s="2" t="inlineStr">
@@ -4539,27 +4539,23 @@
       </c>
       <c r="Q41" s="5" t="inlineStr">
         <is>
-          <t>https://simplify.jobs/p/d07243d2-a109-4f64-a14d-7a75944627e3/Data-Analyst</t>
+          <t>https://targetjobs.co.uk/jobs/consulting-graduate-bristol-september-2027-239989</t>
         </is>
       </c>
       <c r="R41" s="2" t="inlineStr">
         <is>
-          <t>Simplify / Tarve (via web search)</t>
+          <t>TargetJobs (via web search)</t>
         </is>
       </c>
       <c r="S41" s="2" t="inlineStr">
         <is>
-          <t>Updated 8/1/2026; a sponsorship-board copy shows 'apply by 9 September 2026'</t>
-        </is>
-      </c>
-      <c r="T41" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-12</t>
-        </is>
-      </c>
+          <t>No deadline shown</t>
+        </is>
+      </c>
+      <c r="T41" s="2" t="inlineStr"/>
       <c r="U41" s="2" t="inlineStr">
         <is>
-          <t>May already be closed (one copy shows 9 Sep apply-by). Verify on Funding Circle careers.</t>
+          <t>2027 START. Check RSM site for a London/Birmingham consulting variant. Eligibility risk on 'permanent right to work'.</t>
         </is>
       </c>
       <c r="V41" s="6" t="n">
@@ -4578,7 +4574,7 @@
       <c r="C42" s="12" t="n"/>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Barclays (UK)</t>
+          <t>Wise</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -4588,22 +4584,22 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2027 Technology Analyst Graduate Programme</t>
+          <t>Graduate Analyst - London</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Graduate Programme</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>UK (multiple listings)</t>
+          <t>London</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>Aug 2027</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -4612,16 +4608,16 @@
         </is>
       </c>
       <c r="K42" s="2" t="n">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>Graduate technology analyst track in a bank; CS degree plus BA/Jira/Agile experience</t>
+          <t>Graduate analytics role at a fintech; SQL/Python/Power BI dashboarding from your dissertation and ESG dashboard project fit</t>
         </is>
       </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>2025/2026 graduate (Bachelor's/Master's) in data/CS/STEM/economics (per related Wise grad listing)</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr">
@@ -4631,7 +4627,7 @@
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>Accepts applicants who need visa sponsorship</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="P42" s="2" t="inlineStr">
@@ -4641,23 +4637,23 @@
       </c>
       <c r="Q42" s="5" t="inlineStr">
         <is>
-          <t>https://www.gradcracker.com/hub/180/barclays/graduate-job/83373/2027-technology-analyst-graduate-programme</t>
+          <t>https://wise.jobs/job/graduate-analyst-london-in-london-jid-3837</t>
         </is>
       </c>
       <c r="R42" s="2" t="inlineStr">
         <is>
-          <t>Gradcracker (via web search)</t>
+          <t>Web search (wise.jobs / TargetJobs)</t>
         </is>
       </c>
       <c r="S42" s="2" t="inlineStr">
         <is>
-          <t>No closing date in listing excerpt</t>
+          <t>No deadline shown; one Wise grad analyst listing marked 'This vacancy has now expired'</t>
         </is>
       </c>
       <c r="T42" s="2" t="inlineStr"/>
       <c r="U42" s="2" t="inlineStr">
         <is>
-          <t>2027 START. Some tracks are engineering-heavy — pick a business-analysis-oriented role. Verify on company site.</t>
+          <t>Status uncertain — a sister listing has expired; check it is still open. Apply ASAP — may close early.</t>
         </is>
       </c>
       <c r="V42" s="6" t="n">
@@ -4676,17 +4672,17 @@
       <c r="C43" s="12" t="n"/>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>CGI UK</t>
+          <t>India big-tech arms (Google, Microsoft, Amazon [done], Salesforce, Oracle, SAP, Adobe, Cisco, Uber, LinkedIn, ServiceNow, Snowflake, Databricks)</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Technical Graduate - Data Analysis &amp; Data Science 2027</t>
+          <t>Uber — Business Analyst, APAC Analytics &amp; Insights (Hyderabad)</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -4696,30 +4692,30 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>UK (multiple offices)</t>
+          <t>Hyderabad</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Not stated (aggregator estimate ₹5–7 LPA)</t>
         </is>
       </c>
       <c r="K43" s="2" t="n">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>Graduate data-analysis track at a large IT consultancy; SQL/Python/Power BI + CS degree fit</t>
+          <t>0-years-minimum analytics role using SQL/Python/Tableau dashboards and root-cause analysis — your exact stack</t>
         </is>
       </c>
       <c r="M43" s="2" t="inlineStr">
         <is>
-          <t>2:2 and above</t>
+          <t>Graduate, fresher or experienced; SQL, Python, Looker Studio, Tableau</t>
         </is>
       </c>
       <c r="N43" s="2" t="inlineStr">
@@ -4729,7 +4725,7 @@
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>N/A (India)</t>
         </is>
       </c>
       <c r="P43" s="2" t="inlineStr">
@@ -4739,23 +4735,23 @@
       </c>
       <c r="Q43" s="5" t="inlineStr">
         <is>
-          <t>https://www.gradcracker.com/hub/89/cgi/graduate-job/85473/technical-graduate-data-analysis-and-data-science-2027</t>
+          <t>https://jobs.weekday.works/uber-business-analyst</t>
         </is>
       </c>
       <c r="R43" s="2" t="inlineStr">
         <is>
-          <t>Gradcracker (via web search)</t>
+          <t>Weekday / The Muse (via web search)</t>
         </is>
       </c>
       <c r="S43" s="2" t="inlineStr">
         <is>
-          <t>Ongoing</t>
+          <t>No deadline shown</t>
         </is>
       </c>
       <c r="T43" s="2" t="inlineStr"/>
       <c r="U43" s="2" t="inlineStr">
         <is>
-          <t>2027 START. Some CGI roles need UK security clearance — check.</t>
+          <t>Aggregator listing — find the matching posting on uber.com/careers.</t>
         </is>
       </c>
       <c r="V43" s="6" t="n">
@@ -4774,7 +4770,7 @@
       <c r="C44" s="12" t="n"/>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Financial Conduct Authority (FCA)</t>
+          <t>Ebury</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -4784,22 +4780,22 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2027 Regulatory Graduate Programme (London)</t>
+          <t>Graduate Banking Operations Analyst</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Risk</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>London (hybrid, 4 days office)</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -4808,16 +4804,16 @@
         </is>
       </c>
       <c r="K44" s="2" t="n">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>Financial-services regulator grad scheme; FinTech MSc + greenwashing (ESG disclosure) dissertation is directly relevant to FCA conduct/ESG work</t>
+          <t>Graduate operations analyst at an FX/payments fintech; process documentation and stakeholder coordination from your BA case study</t>
         </is>
       </c>
       <c r="M44" s="2" t="inlineStr">
         <is>
-          <t>Graduated or final year; 2:1 (or on track)</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="N44" s="2" t="inlineStr">
@@ -4837,23 +4833,23 @@
       </c>
       <c r="Q44" s="5" t="inlineStr">
         <is>
-          <t>https://www.brightnetwork.co.uk/graduate-jobs/financial-conduct-authority/2027-regulatory-graduate-programme-london</t>
+          <t>https://targetjobs.co.uk/jobs/graduate-banking-operations-analyst-213626</t>
         </is>
       </c>
       <c r="R44" s="2" t="inlineStr">
         <is>
-          <t>Bright Network (via web search)</t>
+          <t>TargetJobs (via web search)</t>
         </is>
       </c>
       <c r="S44" s="2" t="inlineStr">
         <is>
-          <t>Marked 'recently opened'; no closing date in snippet</t>
+          <t>No deadline shown</t>
         </is>
       </c>
       <c r="T44" s="2" t="inlineStr"/>
       <c r="U44" s="2" t="inlineStr">
         <is>
-          <t>2027 START. Mention your greenwashing research (FCA anti-greenwashing rule).</t>
+          <t>Listing may be from an earlier cycle — check it is still open. Role is operational (account opening, mandates).</t>
         </is>
       </c>
       <c r="V44" s="6" t="n">
@@ -4872,7 +4868,7 @@
       <c r="C45" s="12" t="n"/>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Capgemini (UK)</t>
+          <t>Funding Circle</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -4882,40 +4878,40 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Graduate Business Analyst 2027</t>
+          <t>Data Analyst (London, hybrid)</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Not stated (UK)</t>
+          <t>London (hybrid, 3 days office)</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Not stated (Home Office going rate listed as £34,900)</t>
         </is>
       </c>
       <c r="K45" s="2" t="n">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>Explicit graduate BA role; your BRD/BPMN/user-story case study is exactly this work</t>
+          <t>SME-lending fintech data role open to recent grads with strong data skills; SQL/Tableau/Python + CS degree</t>
         </is>
       </c>
       <c r="M45" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Numerical/data degree; 1–2 yrs OR recent graduate with strong data skills; SQL, Tableau</t>
         </is>
       </c>
       <c r="N45" s="2" t="inlineStr">
@@ -4925,33 +4921,37 @@
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Employer holds sponsor licence (listing)</t>
         </is>
       </c>
       <c r="P45" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="Q45" s="5" t="inlineStr">
         <is>
-          <t>https://targetjobs.co.uk/jobs/graduate-business-analyst-2027-249559</t>
+          <t>https://simplify.jobs/p/d07243d2-a109-4f64-a14d-7a75944627e3/Data-Analyst</t>
         </is>
       </c>
       <c r="R45" s="2" t="inlineStr">
         <is>
-          <t>TargetJobs / Gradcracker (via web search)</t>
+          <t>Simplify / Tarve (via web search)</t>
         </is>
       </c>
       <c r="S45" s="2" t="inlineStr">
         <is>
-          <t>No deadline in search result</t>
-        </is>
-      </c>
-      <c r="T45" s="2" t="inlineStr"/>
+          <t>Updated 8/1/2026; a sponsorship-board copy shows 'apply by 9 September 2026'</t>
+        </is>
+      </c>
+      <c r="T45" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
       <c r="U45" s="2" t="inlineStr">
         <is>
-          <t>2027 START. Gradcracker files it under Capgemini Engineering. Location not stated. Verify on company site.</t>
+          <t>May already be closed (one copy shows 9 Sep apply-by). Verify on Funding Circle careers.</t>
         </is>
       </c>
       <c r="V45" s="6" t="n">
@@ -4970,7 +4970,7 @@
       <c r="C46" s="12" t="n"/>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>TCS (Tata Consultancy Services)</t>
+          <t>Barclays (UK)</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -4980,7 +4980,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>TCS UK Graduate Programme — Business Analyst track</t>
+          <t>2027 Technology Analyst Graduate Programme</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -4990,12 +4990,12 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>UK (location not stated)</t>
+          <t>UK (multiple listings)</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Aug 2027</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -5004,16 +5004,16 @@
         </is>
       </c>
       <c r="K46" s="2" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>Year-round UK grad intake with a BA role; CS degree (2:1) + BA case study fit the stated technology-degree requirement</t>
+          <t>Graduate technology analyst track in a bank; CS degree plus BA/Jira/Agile experience</t>
         </is>
       </c>
       <c r="M46" s="2" t="inlineStr">
         <is>
-          <t>2:1 or better in a technology/IT/CS-related subject</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="N46" s="2" t="inlineStr">
@@ -5023,33 +5023,33 @@
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Accepts applicants who need visa sponsorship</t>
         </is>
       </c>
       <c r="P46" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="Q46" s="5" t="inlineStr">
         <is>
-          <t>https://careerforfreshers.com/jobs/tcs-graduate-opportunities-for-fresher-analyst-engineer-0-1-yrs-uk-europe/</t>
+          <t>https://www.gradcracker.com/hub/180/barclays/graduate-job/83373/2027-technology-analyst-graduate-programme</t>
         </is>
       </c>
       <c r="R46" s="2" t="inlineStr">
         <is>
-          <t>Web search (practiceaptitudetests / careerforfreshers)</t>
+          <t>Gradcracker (via web search)</t>
         </is>
       </c>
       <c r="S46" s="2" t="inlineStr">
         <is>
-          <t>Graduate programme can be applied for year-round</t>
+          <t>No closing date in listing excerpt</t>
         </is>
       </c>
       <c r="T46" s="2" t="inlineStr"/>
       <c r="U46" s="2" t="inlineStr">
         <is>
-          <t>Aggregator sources only — find the live UK posting on tcs.com/careers before applying.</t>
+          <t>2027 START. Some tracks are engineering-heavy — pick a business-analysis-oriented role. Verify on company site.</t>
         </is>
       </c>
       <c r="V46" s="6" t="n">
@@ -5068,7 +5068,7 @@
       <c r="C47" s="12" t="n"/>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Arup</t>
+          <t>CGI UK</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -5078,17 +5078,17 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Graduate Sustainability Consultant 2027</t>
+          <t>Technical Graduate - Data Analysis &amp; Data Science 2027</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>ESG</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>North UK (Scotland, NI, northern England)</t>
+          <t>UK (multiple offices)</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
@@ -5102,16 +5102,16 @@
         </is>
       </c>
       <c r="K47" s="2" t="n">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>GHG/sustainability performance data analysis; greenwashing dissertation + ESG dashboard + net-zero MCC project</t>
+          <t>Graduate data-analysis track at a large IT consultancy; SQL/Python/Power BI + CS degree fit</t>
         </is>
       </c>
       <c r="M47" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>2:2 and above</t>
         </is>
       </c>
       <c r="N47" s="2" t="inlineStr">
@@ -5121,7 +5121,7 @@
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>Unable to offer visa sponsorship</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="P47" s="2" t="inlineStr">
@@ -5131,23 +5131,23 @@
       </c>
       <c r="Q47" s="5" t="inlineStr">
         <is>
-          <t>https://www.brightnetwork.co.uk/graduate-jobs/arup/graduate-sustainability-consultant-2027-1</t>
+          <t>https://www.gradcracker.com/hub/89/cgi/graduate-job/85473/technical-graduate-data-analysis-and-data-science-2027</t>
         </is>
       </c>
       <c r="R47" s="2" t="inlineStr">
         <is>
-          <t>Bright Network / Gradcracker (via web search)</t>
+          <t>Gradcracker (via web search)</t>
         </is>
       </c>
       <c r="S47" s="2" t="inlineStr">
         <is>
-          <t>Early application recommended</t>
+          <t>Ongoing</t>
         </is>
       </c>
       <c r="T47" s="2" t="inlineStr"/>
       <c r="U47" s="2" t="inlineStr">
         <is>
-          <t>2027 START. Apply ASAP — may close early.</t>
+          <t>2027 START. Some CGI roles need UK security clearance — check.</t>
         </is>
       </c>
       <c r="V47" s="6" t="n">
@@ -5166,32 +5166,32 @@
       <c r="C48" s="12" t="n"/>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Citigroup (UK)</t>
+          <t>India big-tech arms (Google, Microsoft, Amazon [done], Salesforce, Oracle, SAP, Adobe, Cisco, Uber, LinkedIn, ServiceNow, Snowflake, Databricks)</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Banking, Commercial Banking, Full Time Analyst, London - United Kingdom 2027</t>
+          <t>Oracle — Business Analyst (Bengaluru)</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Graduate Programme</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Bengaluru (on-site)</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>Jul 2027</t>
+          <t>ASAP</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
@@ -5200,56 +5200,52 @@
         </is>
       </c>
       <c r="K48" s="2" t="n">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>Graduate analyst programme with credit/financial analysis; Excel financial modelling and FinTech MSc fit</t>
+          <t>Requirements gathering, data validation and root-cause analysis — maps to your BA case study and SQL</t>
         </is>
       </c>
       <c r="M48" s="2" t="inlineStr">
         <is>
-          <t>2:1 at undergraduate level; penultimate/final-year wording in listing</t>
+          <t>0 to 2+ years experience</t>
         </is>
       </c>
       <c r="N48" s="2" t="inlineStr">
         <is>
-          <t>Starts with in-depth training</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>N/A (India)</t>
         </is>
       </c>
       <c r="P48" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="Q48" s="5" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/job/london/banking-commercial-banking-full-time-analyst-london-united-kingdom-2027/287/100996355040</t>
+          <t>https://nxtwave-join.prosple.com/graduate-employers/oracle-india/jobs-internships/business-analyst-0</t>
         </is>
       </c>
       <c r="R48" s="2" t="inlineStr">
         <is>
-          <t>Web search (jobs.citi.com)</t>
+          <t>Prosple (via web search)</t>
         </is>
       </c>
       <c r="S48" s="2" t="inlineStr">
         <is>
-          <t>No deadline shown; posted 22 Sep 2026</t>
-        </is>
-      </c>
-      <c r="T48" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
+          <t>Start ASAP; no deadline</t>
+        </is>
+      </c>
+      <c r="T48" s="2" t="inlineStr"/>
       <c r="U48" s="2" t="inlineStr">
         <is>
-          <t>2027 START. Listing mentions final-year students — confirm graduates are eligible. Apply ASAP — may close early.</t>
+          <t>Verify still open on Oracle careers.</t>
         </is>
       </c>
       <c r="V48" s="6" t="n">
@@ -5268,7 +5264,7 @@
       <c r="C49" s="12" t="n"/>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Goldman Sachs (UK)</t>
+          <t>Financial Conduct Authority (FCA)</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -5278,12 +5274,12 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2027 EMEA New Analyst Programme (London)</t>
+          <t>2027 Regulatory Graduate Programme (London)</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Graduate Programme</t>
+          <t>Risk</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -5293,7 +5289,7 @@
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>Summer 2027</t>
+          <t>2027</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
@@ -5302,16 +5298,16 @@
         </is>
       </c>
       <c r="K49" s="2" t="n">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>Full-time graduate analyst programme; choose a division such as Operations / Risk / Engineering-adjacent analytics to match your data background</t>
+          <t>Financial-services regulator grad scheme; FinTech MSc + greenwashing (ESG disclosure) dissertation is directly relevant to FCA conduct/ESG work</t>
         </is>
       </c>
       <c r="M49" s="2" t="inlineStr">
         <is>
-          <t>Graduating Dec 2026 – Jul 2027 (per Americas equivalent)</t>
+          <t>Graduated or final year; 2:1 (or on track)</t>
         </is>
       </c>
       <c r="N49" s="2" t="inlineStr">
@@ -5326,28 +5322,28 @@
       </c>
       <c r="P49" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="Q49" s="5" t="inlineStr">
         <is>
-          <t>https://higher.gs.com/</t>
+          <t>https://www.brightnetwork.co.uk/graduate-jobs/financial-conduct-authority/2027-regulatory-graduate-programme-london</t>
         </is>
       </c>
       <c r="R49" s="2" t="inlineStr">
         <is>
-          <t>Web search (aggregators)</t>
+          <t>Bright Network (via web search)</t>
         </is>
       </c>
       <c r="S49" s="2" t="inlineStr">
         <is>
-          <t>Application timelines vary according to the business</t>
+          <t>Marked 'recently opened'; no closing date in snippet</t>
         </is>
       </c>
       <c r="T49" s="2" t="inlineStr"/>
       <c r="U49" s="2" t="inlineStr">
         <is>
-          <t>2027 START. Deadlines differ by division — some may have closed. Verify on higher.gs.com.</t>
+          <t>2027 START. Mention your greenwashing research (FCA anti-greenwashing rule).</t>
         </is>
       </c>
       <c r="V49" s="6" t="n">
@@ -5366,7 +5362,7 @@
       <c r="C50" s="12" t="n"/>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>BNY (Mellon)</t>
+          <t>Capgemini (UK)</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -5376,17 +5372,17 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2027 BNY Analyst Program - Risk and Compliance (London)</t>
+          <t>Graduate Business Analyst 2027</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Risk</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Not stated (UK)</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
@@ -5400,16 +5396,16 @@
         </is>
       </c>
       <c r="K50" s="2" t="n">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>Graduate risk analyst track; accepts Dec 2026 graduates — your MSc award may fall in that window</t>
+          <t>Explicit graduate BA role; your BRD/BPMN/user-story case study is exactly this work</t>
         </is>
       </c>
       <c r="M50" s="2" t="inlineStr">
         <is>
-          <t>Graduating 2027 or Dec 2026; 2:1 on track</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="N50" s="2" t="inlineStr">
@@ -5419,7 +5415,7 @@
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>Must not require sponsorship now or in the future</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="P50" s="2" t="inlineStr">
@@ -5429,12 +5425,12 @@
       </c>
       <c r="Q50" s="5" t="inlineStr">
         <is>
-          <t>https://targetjobs.co.uk/jobs/2027-bny-analyst-program-risk-and-compliance-london-249629</t>
+          <t>https://targetjobs.co.uk/jobs/graduate-business-analyst-2027-249559</t>
         </is>
       </c>
       <c r="R50" s="2" t="inlineStr">
         <is>
-          <t>TargetJobs (via web search)</t>
+          <t>TargetJobs / Gradcracker (via web search)</t>
         </is>
       </c>
       <c r="S50" s="2" t="inlineStr">
@@ -5445,7 +5441,7 @@
       <c r="T50" s="2" t="inlineStr"/>
       <c r="U50" s="2" t="inlineStr">
         <is>
-          <t>2027 START. Sponsorship restriction — Graduate visa may not satisfy 'in the future' clause. Verify on company site.</t>
+          <t>2027 START. Gradcracker files it under Capgemini Engineering. Location not stated. Verify on company site.</t>
         </is>
       </c>
       <c r="V50" s="6" t="n">
@@ -5464,7 +5460,7 @@
       <c r="C51" s="12" t="n"/>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>RSM UK</t>
+          <t>TCS (Tata Consultancy Services)</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -5474,22 +5470,22 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Technology Audit Specialist Graduate - Birmingham - September 2027</t>
+          <t>TCS UK Graduate Programme — Business Analyst track</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Risk</t>
+          <t>Graduate Programme</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>Birmingham (also London listing)</t>
+          <t>UK (location not stated)</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>Sep 2027</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr">
@@ -5498,16 +5494,16 @@
         </is>
       </c>
       <c r="K51" s="2" t="n">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>IT risk/assurance grad in Birmingham; CS degree + network-analyst internships fit tech-controls work</t>
+          <t>Year-round UK grad intake with a BA role; CS degree (2:1) + BA case study fit the stated technology-degree requirement</t>
         </is>
       </c>
       <c r="M51" s="2" t="inlineStr">
         <is>
-          <t>Not stated; CISA sponsored after ~2 years</t>
+          <t>2:1 or better in a technology/IT/CS-related subject</t>
         </is>
       </c>
       <c r="N51" s="2" t="inlineStr">
@@ -5527,23 +5523,23 @@
       </c>
       <c r="Q51" s="5" t="inlineStr">
         <is>
-          <t>https://targetjobs.co.uk/jobs/technology-audit-specialist-graduate-birmingham-september-2027-240093</t>
+          <t>https://careerforfreshers.com/jobs/tcs-graduate-opportunities-for-fresher-analyst-engineer-0-1-yrs-uk-europe/</t>
         </is>
       </c>
       <c r="R51" s="2" t="inlineStr">
         <is>
-          <t>TargetJobs (via web search)</t>
+          <t>Web search (practiceaptitudetests / careerforfreshers)</t>
         </is>
       </c>
       <c r="S51" s="2" t="inlineStr">
         <is>
-          <t>No deadline shown</t>
+          <t>Graduate programme can be applied for year-round</t>
         </is>
       </c>
       <c r="T51" s="2" t="inlineStr"/>
       <c r="U51" s="2" t="inlineStr">
         <is>
-          <t>2027 START. Birmingham bonus.</t>
+          <t>Aggregator sources only — find the live UK posting on tcs.com/careers before applying.</t>
         </is>
       </c>
       <c r="V51" s="6" t="n">
@@ -5562,7 +5558,7 @@
       <c r="C52" s="12" t="n"/>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>Arup</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -5572,17 +5568,17 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Shell Graduate Programme 2027 (Commercial / Finance / Information Digital Technologies pathways)</t>
+          <t>Graduate Sustainability Consultant 2027</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Graduate Programme</t>
+          <t>ESG</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>UK (London)</t>
+          <t>North UK (Scotland, NI, northern England)</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
@@ -5596,26 +5592,26 @@
         </is>
       </c>
       <c r="K52" s="2" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>Energy-transition major's grad programme; you meet the UK-degree + within-3-years rule; ESG/net-zero work fits Commercial/IDT tracks</t>
+          <t>GHG/sustainability performance data analysis; greenwashing dissertation + ESG dashboard + net-zero MCC project</t>
         </is>
       </c>
       <c r="M52" s="2" t="inlineStr">
         <is>
-          <t>UK Bachelor's/Master's; graduating 2027 or within last 3 years; live in UK</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="N52" s="2" t="inlineStr">
         <is>
-          <t>Virtual Job Try-out → on-demand interview → case study &amp; interview</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Unable to offer visa sponsorship</t>
         </is>
       </c>
       <c r="P52" s="2" t="inlineStr">
@@ -5625,17 +5621,17 @@
       </c>
       <c r="Q52" s="5" t="inlineStr">
         <is>
-          <t>https://www.shell.co.uk/careers/students-and-graduates.html</t>
+          <t>https://www.brightnetwork.co.uk/graduate-jobs/arup/graduate-sustainability-consultant-2027-1</t>
         </is>
       </c>
       <c r="R52" s="2" t="inlineStr">
         <is>
-          <t>Company site + aggregator (via web search)</t>
+          <t>Bright Network / Gradcracker (via web search)</t>
         </is>
       </c>
       <c r="S52" s="2" t="inlineStr">
         <is>
-          <t>Opened Sep 2026; previous cycle closed 10 Dec 2025; rolling, may close earlier</t>
+          <t>Early application recommended</t>
         </is>
       </c>
       <c r="T52" s="2" t="inlineStr"/>
@@ -5660,7 +5656,7 @@
       <c r="C53" s="12" t="n"/>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Tesco</t>
+          <t>Citigroup (UK)</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -5670,45 +5666,45 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>IMS Customer Propositions Graduate Scheme</t>
+          <t>Banking, Commercial Banking, Full Time Analyst, London - United Kingdom 2027</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Graduate Programme</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>Edinburgh / Glasgow</t>
+          <t>London</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>Sep 2027</t>
+          <t>Jul 2027</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>£32,000</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="K53" s="2" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="L53" s="2" t="inlineStr">
         <is>
-          <t>Customer-insight grad scheme accepting analytics &amp; data-science disciplines; Python/SQL/Power BI</t>
+          <t>Graduate analyst programme with credit/financial analysis; Excel financial modelling and FinTech MSc fit</t>
         </is>
       </c>
       <c r="M53" s="2" t="inlineStr">
         <is>
-          <t>Analytics / data science among accepted disciplines</t>
+          <t>2:1 at undergraduate level; penultimate/final-year wording in listing</t>
         </is>
       </c>
       <c r="N53" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Starts with in-depth training</t>
         </is>
       </c>
       <c r="O53" s="2" t="inlineStr">
@@ -5718,28 +5714,32 @@
       </c>
       <c r="P53" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="Q53" s="5" t="inlineStr">
         <is>
-          <t>https://www.gradcracker.com/hub/848/tesco/graduate-job/83879/ims-customer-propositions-graduate-scheme</t>
+          <t>https://jobs.citi.com/job/london/banking-commercial-banking-full-time-analyst-london-united-kingdom-2027/287/100996355040</t>
         </is>
       </c>
       <c r="R53" s="2" t="inlineStr">
         <is>
-          <t>Gradcracker (via web search)</t>
+          <t>Web search (jobs.citi.com)</t>
         </is>
       </c>
       <c r="S53" s="2" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="T53" s="2" t="inlineStr"/>
+          <t>No deadline shown; posted 22 Sep 2026</t>
+        </is>
+      </c>
+      <c r="T53" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="U53" s="2" t="inlineStr">
         <is>
-          <t>2027 START.</t>
+          <t>2027 START. Listing mentions final-year students — confirm graduates are eligible. Apply ASAP — may close early.</t>
         </is>
       </c>
       <c r="V53" s="6" t="n">
@@ -5758,7 +5758,7 @@
       <c r="C54" s="12" t="n"/>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Allica Bank</t>
+          <t>Goldman Sachs (UK)</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -5768,12 +5768,12 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst - 8 Month FTC</t>
+          <t>2027 EMEA New Analyst Programme (London)</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Graduate Programme</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Summer 2027</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
@@ -5792,16 +5792,16 @@
         </is>
       </c>
       <c r="K54" s="2" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>Fintech bank data role across Finance, Ops, Credit Risk and Product; SQL/Python/Power BI fit; fixed-term can be a foot in the door</t>
+          <t>Full-time graduate analyst programme; choose a division such as Operations / Risk / Engineering-adjacent analytics to match your data background</t>
         </is>
       </c>
       <c r="M54" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Graduating Dec 2026 – Jul 2027 (per Americas equivalent)</t>
         </is>
       </c>
       <c r="N54" s="2" t="inlineStr">
@@ -5816,32 +5816,28 @@
       </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="Q54" s="5" t="inlineStr">
         <is>
-          <t>https://portfoliojobs.tcv.com/companies/allica-bank-2/jobs/92626603-data-analyst-8-month-ftc</t>
+          <t>https://higher.gs.com/</t>
         </is>
       </c>
       <c r="R54" s="2" t="inlineStr">
         <is>
-          <t>TCV portfolio jobs (via web search)</t>
+          <t>Web search (aggregators)</t>
         </is>
       </c>
       <c r="S54" s="2" t="inlineStr">
         <is>
-          <t>Posted Sep 9, 2026; no deadline</t>
-        </is>
-      </c>
-      <c r="T54" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
+          <t>Application timelines vary according to the business</t>
+        </is>
+      </c>
+      <c r="T54" s="2" t="inlineStr"/>
       <c r="U54" s="2" t="inlineStr">
         <is>
-          <t>8-month fixed-term contract. Seniority not stated.</t>
+          <t>2027 START. Deadlines differ by division — some may have closed. Verify on higher.gs.com.</t>
         </is>
       </c>
       <c r="V54" s="6" t="n">
@@ -5860,7 +5856,7 @@
       <c r="C55" s="12" t="n"/>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Salesforce (UK)</t>
+          <t>BNY (Mellon)</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -5870,22 +5866,22 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Associate Analyst, Sales Strategy &amp; Operations (Futureforce) — London</t>
+          <t>2027 BNY Analyst Program - Risk and Compliance (London)</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>Risk</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>London (onsite)</t>
+          <t>London</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>2027</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr">
@@ -5894,16 +5890,16 @@
         </is>
       </c>
       <c r="K55" s="2" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="L55" s="2" t="inlineStr">
         <is>
-          <t>Futureforce early-career strategy/ops analyst; KPI definition and data-driven recommendations from your ESG dashboard project</t>
+          <t>Graduate risk analyst track; accepts Dec 2026 graduates — your MSc award may fall in that window</t>
         </is>
       </c>
       <c r="M55" s="2" t="inlineStr">
         <is>
-          <t>Data-driven recommendations to UK&amp;I senior leaders</t>
+          <t>Graduating 2027 or Dec 2026; 2:1 on track</t>
         </is>
       </c>
       <c r="N55" s="2" t="inlineStr">
@@ -5913,37 +5909,33 @@
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Must not require sponsorship now or in the future</t>
         </is>
       </c>
       <c r="P55" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="Q55" s="5" t="inlineStr">
         <is>
-          <t>https://www.themuse.com/jobs/salesforce/associate-analyst-sales-strategy-operations-b91a77</t>
+          <t>https://targetjobs.co.uk/jobs/2027-bny-analyst-program-risk-and-compliance-london-249629</t>
         </is>
       </c>
       <c r="R55" s="2" t="inlineStr">
         <is>
-          <t>Web search (The Muse / EuroTopTech)</t>
+          <t>TargetJobs (via web search)</t>
         </is>
       </c>
       <c r="S55" s="2" t="inlineStr">
         <is>
-          <t>Posted July 2026; no deadline shown</t>
-        </is>
-      </c>
-      <c r="T55" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+          <t>No deadline in search result</t>
+        </is>
+      </c>
+      <c r="T55" s="2" t="inlineStr"/>
       <c r="U55" s="2" t="inlineStr">
         <is>
-          <t>Aggregator labels it mid-level — confirm entry-level on Salesforce careers. Posted ~July 2026; may be filled.</t>
+          <t>2027 START. Sponsorship restriction — Graduate visa may not satisfy 'in the future' clause. Verify on company site.</t>
         </is>
       </c>
       <c r="V55" s="6" t="n">
@@ -5962,7 +5954,7 @@
       <c r="C56" s="12" t="n"/>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Jacobs</t>
+          <t>RSM UK</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -5972,17 +5964,17 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Graduate Sustainability Consultant - Leeds 2027</t>
+          <t>Technology Audit Specialist Graduate - Birmingham - September 2027</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>ESG</t>
+          <t>Risk</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Leeds</t>
+          <t>Birmingham (also London listing)</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
@@ -5996,16 +5988,16 @@
         </is>
       </c>
       <c r="K56" s="2" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>Sustainability consulting grad; ESG dissertation + net-zero MCC</t>
+          <t>IT risk/assurance grad in Birmingham; CS degree + network-analyst internships fit tech-controls work</t>
         </is>
       </c>
       <c r="M56" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Not stated; CISA sponsored after ~2 years</t>
         </is>
       </c>
       <c r="N56" s="2" t="inlineStr">
@@ -6025,23 +6017,23 @@
       </c>
       <c r="Q56" s="5" t="inlineStr">
         <is>
-          <t>https://www.brightnetwork.co.uk/graduate-jobs/jacobs/graduate-sustainability-consultant-leeds-2027-am4u</t>
+          <t>https://targetjobs.co.uk/jobs/technology-audit-specialist-graduate-birmingham-september-2027-240093</t>
         </is>
       </c>
       <c r="R56" s="2" t="inlineStr">
         <is>
-          <t>Bright Network (via web search)</t>
+          <t>TargetJobs (via web search)</t>
         </is>
       </c>
       <c r="S56" s="2" t="inlineStr">
         <is>
-          <t>No closing date shown</t>
+          <t>No deadline shown</t>
         </is>
       </c>
       <c r="T56" s="2" t="inlineStr"/>
       <c r="U56" s="2" t="inlineStr">
         <is>
-          <t>2027 START.</t>
+          <t>2027 START. Birmingham bonus.</t>
         </is>
       </c>
       <c r="V56" s="6" t="n">
@@ -6060,7 +6052,7 @@
       <c r="C57" s="12" t="n"/>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Tesco</t>
+          <t>Shell</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -6070,45 +6062,45 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Technology - Product Management Graduate Scheme</t>
+          <t>Shell Graduate Programme 2027 (Commercial / Finance / Information Digital Technologies pathways)</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>FinTech</t>
+          <t>Graduate Programme</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>Welwyn Garden City</t>
+          <t>UK (London)</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>Sep 2027</t>
+          <t>2027</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>£40,000</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="K57" s="2" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="L57" s="2" t="inlineStr">
         <is>
-          <t>Product grad scheme accepting analytics/data-science grads; user stories, Jira and requirements work from your BA case study</t>
+          <t>Energy-transition major's grad programme; you meet the UK-degree + within-3-years rule; ESG/net-zero work fits Commercial/IDT tracks</t>
         </is>
       </c>
       <c r="M57" s="2" t="inlineStr">
         <is>
-          <t>Accepts analytics/statistics and data science graduates</t>
+          <t>UK Bachelor's/Master's; graduating 2027 or within last 3 years; live in UK</t>
         </is>
       </c>
       <c r="N57" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Virtual Job Try-out → on-demand interview → case study &amp; interview</t>
         </is>
       </c>
       <c r="O57" s="2" t="inlineStr">
@@ -6123,23 +6115,23 @@
       </c>
       <c r="Q57" s="5" t="inlineStr">
         <is>
-          <t>https://www.gradcracker.com/hub/848/tesco/graduate-job/83546/technology-product-management-graduate-scheme</t>
+          <t>https://www.shell.co.uk/careers/students-and-graduates.html</t>
         </is>
       </c>
       <c r="R57" s="2" t="inlineStr">
         <is>
-          <t>Gradcracker (via web search)</t>
+          <t>Company site + aggregator (via web search)</t>
         </is>
       </c>
       <c r="S57" s="2" t="inlineStr">
         <is>
-          <t>Ongoing</t>
+          <t>Opened Sep 2026; previous cycle closed 10 Dec 2025; rolling, may close earlier</t>
         </is>
       </c>
       <c r="T57" s="2" t="inlineStr"/>
       <c r="U57" s="2" t="inlineStr">
         <is>
-          <t>2027 START.</t>
+          <t>2027 START. Apply ASAP — may close early.</t>
         </is>
       </c>
       <c r="V57" s="6" t="n">
@@ -6158,7 +6150,7 @@
       <c r="C58" s="12" t="n"/>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Moody's</t>
+          <t>Tesco</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -6168,40 +6160,40 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Moody's Insurance Solutions Graduate Program - Cyber and Casualty</t>
+          <t>IMS Customer Propositions Graduate Scheme</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Risk</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Edinburgh / Glasgow</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Sep 2027</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>£32,000</t>
         </is>
       </c>
       <c r="K58" s="2" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="L58" s="2" t="inlineStr">
         <is>
-          <t>Graduate risk-analytics programme at a ratings/risk firm; quantitative modelling from your econometrics work applies</t>
+          <t>Customer-insight grad scheme accepting analytics &amp; data-science disciplines; Python/SQL/Power BI</t>
         </is>
       </c>
       <c r="M58" s="2" t="inlineStr">
         <is>
-          <t>Not stated</t>
+          <t>Analytics / data science among accepted disciplines</t>
         </is>
       </c>
       <c r="N58" s="2" t="inlineStr">
@@ -6216,32 +6208,28 @@
       </c>
       <c r="P58" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="Q58" s="5" t="inlineStr">
         <is>
-          <t>https://careers.moodys.com/en/job/london/moody-s-insurance-solutions-graduate-program-cyber-and-casualty/49841/97200112128</t>
+          <t>https://www.gradcracker.com/hub/848/tesco/graduate-job/83879/ims-customer-propositions-graduate-scheme</t>
         </is>
       </c>
       <c r="R58" s="2" t="inlineStr">
         <is>
-          <t>Web search (careers.moodys.com)</t>
+          <t>Gradcracker (via web search)</t>
         </is>
       </c>
       <c r="S58" s="2" t="inlineStr">
         <is>
-          <t>Posted 07/01/2026; no deadline shown</t>
-        </is>
-      </c>
-      <c r="T58" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="T58" s="2" t="inlineStr"/>
       <c r="U58" s="2" t="inlineStr">
         <is>
-          <t>Start date not stated; verify still open.</t>
+          <t>2027 START.</t>
         </is>
       </c>
       <c r="V58" s="6" t="n">
@@ -6260,7 +6248,7 @@
       <c r="C59" s="12" t="n"/>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Jacobs</t>
+          <t>Allica Bank</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -6270,22 +6258,22 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Graduate Risk Manager</t>
+          <t>Data Analyst - 8 Month FTC</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Risk</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>London</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>Sep 2027</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr">
@@ -6294,16 +6282,16 @@
         </is>
       </c>
       <c r="K59" s="2" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="L59" s="2" t="inlineStr">
         <is>
-          <t>Project risk analytics grad; Data Science/Analytics backgrounds welcome; econometrics + Python</t>
+          <t>Fintech bank data role across Finance, Ops, Credit Risk and Product; SQL/Python/Power BI fit; fixed-term can be a foot in the door</t>
         </is>
       </c>
       <c r="M59" s="2" t="inlineStr">
         <is>
-          <t>Construction, Data Science, Maths, Analytics degrees</t>
+          <t>Not stated</t>
         </is>
       </c>
       <c r="N59" s="2" t="inlineStr">
@@ -6323,31 +6311,533 @@
       </c>
       <c r="Q59" s="5" t="inlineStr">
         <is>
-          <t>https://www.gradcracker.com/hub/41/jacobs/graduate-job/83471/graduate-risk-manager</t>
+          <t>https://portfoliojobs.tcv.com/companies/allica-bank-2/jobs/92626603-data-analyst-8-month-ftc</t>
         </is>
       </c>
       <c r="R59" s="2" t="inlineStr">
         <is>
-          <t>Gradcracker (via web search)</t>
+          <t>TCV portfolio jobs (via web search)</t>
         </is>
       </c>
       <c r="S59" s="2" t="inlineStr">
         <is>
-          <t>No closing date shown</t>
-        </is>
-      </c>
-      <c r="T59" s="2" t="inlineStr"/>
+          <t>Posted Sep 9, 2026; no deadline</t>
+        </is>
+      </c>
+      <c r="T59" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="U59" s="2" t="inlineStr">
         <is>
-          <t>2027 START.</t>
+          <t>8-month fixed-term contract. Seniority not stated.</t>
         </is>
       </c>
       <c r="V59" s="6" t="n">
         <v>46307</v>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="11" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="C60" s="12" t="n"/>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Salesforce (UK)</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>Associate Analyst, Sales Strategy &amp; Operations (Futureforce) — London</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Business Analyst</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>London (onsite)</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>Futureforce early-career strategy/ops analyst; KPI definition and data-driven recommendations from your ESG dashboard project</t>
+        </is>
+      </c>
+      <c r="M60" s="2" t="inlineStr">
+        <is>
+          <t>Data-driven recommendations to UK&amp;I senior leaders</t>
+        </is>
+      </c>
+      <c r="N60" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="O60" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="P60" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q60" s="5" t="inlineStr">
+        <is>
+          <t>https://www.themuse.com/jobs/salesforce/associate-analyst-sales-strategy-operations-b91a77</t>
+        </is>
+      </c>
+      <c r="R60" s="2" t="inlineStr">
+        <is>
+          <t>Web search (The Muse / EuroTopTech)</t>
+        </is>
+      </c>
+      <c r="S60" s="2" t="inlineStr">
+        <is>
+          <t>Posted July 2026; no deadline shown</t>
+        </is>
+      </c>
+      <c r="T60" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="U60" s="2" t="inlineStr">
+        <is>
+          <t>Aggregator labels it mid-level — confirm entry-level on Salesforce careers. Posted ~July 2026; may be filled.</t>
+        </is>
+      </c>
+      <c r="V60" s="6" t="n">
+        <v>46307</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="11" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="C61" s="12" t="n"/>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Jacobs</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>Graduate Sustainability Consultant - Leeds 2027</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>ESG</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>Leeds</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>Sep 2027</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>Sustainability consulting grad; ESG dissertation + net-zero MCC</t>
+        </is>
+      </c>
+      <c r="M61" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="N61" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="O61" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="P61" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q61" s="5" t="inlineStr">
+        <is>
+          <t>https://www.brightnetwork.co.uk/graduate-jobs/jacobs/graduate-sustainability-consultant-leeds-2027-am4u</t>
+        </is>
+      </c>
+      <c r="R61" s="2" t="inlineStr">
+        <is>
+          <t>Bright Network (via web search)</t>
+        </is>
+      </c>
+      <c r="S61" s="2" t="inlineStr">
+        <is>
+          <t>No closing date shown</t>
+        </is>
+      </c>
+      <c r="T61" s="2" t="inlineStr"/>
+      <c r="U61" s="2" t="inlineStr">
+        <is>
+          <t>2027 START.</t>
+        </is>
+      </c>
+      <c r="V61" s="6" t="n">
+        <v>46307</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="11" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="C62" s="12" t="n"/>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Tesco</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>Technology - Product Management Graduate Scheme</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>FinTech</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>Welwyn Garden City</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>Sep 2027</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>£40,000</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>Product grad scheme accepting analytics/data-science grads; user stories, Jira and requirements work from your BA case study</t>
+        </is>
+      </c>
+      <c r="M62" s="2" t="inlineStr">
+        <is>
+          <t>Accepts analytics/statistics and data science graduates</t>
+        </is>
+      </c>
+      <c r="N62" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="O62" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="P62" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q62" s="5" t="inlineStr">
+        <is>
+          <t>https://www.gradcracker.com/hub/848/tesco/graduate-job/83546/technology-product-management-graduate-scheme</t>
+        </is>
+      </c>
+      <c r="R62" s="2" t="inlineStr">
+        <is>
+          <t>Gradcracker (via web search)</t>
+        </is>
+      </c>
+      <c r="S62" s="2" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="T62" s="2" t="inlineStr"/>
+      <c r="U62" s="2" t="inlineStr">
+        <is>
+          <t>2027 START.</t>
+        </is>
+      </c>
+      <c r="V62" s="6" t="n">
+        <v>46307</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="11" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="C63" s="12" t="n"/>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Moody's</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>Moody's Insurance Solutions Graduate Program - Cyber and Casualty</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="K63" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>Graduate risk-analytics programme at a ratings/risk firm; quantitative modelling from your econometrics work applies</t>
+        </is>
+      </c>
+      <c r="M63" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="N63" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="O63" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="P63" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q63" s="5" t="inlineStr">
+        <is>
+          <t>https://careers.moodys.com/en/job/london/moody-s-insurance-solutions-graduate-program-cyber-and-casualty/49841/97200112128</t>
+        </is>
+      </c>
+      <c r="R63" s="2" t="inlineStr">
+        <is>
+          <t>Web search (careers.moodys.com)</t>
+        </is>
+      </c>
+      <c r="S63" s="2" t="inlineStr">
+        <is>
+          <t>Posted 07/01/2026; no deadline shown</t>
+        </is>
+      </c>
+      <c r="T63" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="U63" s="2" t="inlineStr">
+        <is>
+          <t>Start date not stated; verify still open.</t>
+        </is>
+      </c>
+      <c r="V63" s="6" t="n">
+        <v>46307</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="11" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="C64" s="12" t="n"/>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Jacobs</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>Graduate Risk Manager</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>Sep 2027</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>Project risk analytics grad; Data Science/Analytics backgrounds welcome; econometrics + Python</t>
+        </is>
+      </c>
+      <c r="M64" s="2" t="inlineStr">
+        <is>
+          <t>Construction, Data Science, Maths, Analytics degrees</t>
+        </is>
+      </c>
+      <c r="N64" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="O64" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="P64" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q64" s="5" t="inlineStr">
+        <is>
+          <t>https://www.gradcracker.com/hub/41/jacobs/graduate-job/83471/graduate-risk-manager</t>
+        </is>
+      </c>
+      <c r="R64" s="2" t="inlineStr">
+        <is>
+          <t>Gradcracker (via web search)</t>
+        </is>
+      </c>
+      <c r="S64" s="2" t="inlineStr">
+        <is>
+          <t>No closing date shown</t>
+        </is>
+      </c>
+      <c r="T64" s="2" t="inlineStr"/>
+      <c r="U64" s="2" t="inlineStr">
+        <is>
+          <t>2027 START.</t>
+        </is>
+      </c>
+      <c r="V64" s="6" t="n">
+        <v>46307</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:V59"/>
+  <autoFilter ref="A1:V64"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -6407,6 +6897,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId63"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7333,7 +7828,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -7973,17 +8468,17 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>WTW (Willis Towers Watson)</t>
+          <t>SBI (State Bank of India)</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>2027 Retirement Actuarial Graduate Trainee Consultant Programme</t>
+          <t>SBI Probationary Officer 2026</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -7993,24 +8488,24 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>https://www.gradcracker.com/hub/294/wtw/graduate-job/82421/2027-retirement-actuarial-graduate-trainee-consultant-programme</t>
+          <t>https://www.freepressjournal.in/education/sbi-po-recruitment-2026-last-date-to-apply-tomorrow-for-1500-probationary-officer-posts</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>BDO UK</t>
+          <t>WTW (Willis Towers Watson)</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>2027 Associate Management Graduate Programme - London (Consulting)</t>
+          <t>2027 Retirement Actuarial Graduate Trainee Consultant Programme</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -8020,35 +8515,62 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>https://targetjobs.co.uk/jobs/2027-associate-management-graduate-programme-london-245547</t>
+          <t>https://www.gradcracker.com/hub/294/wtw/graduate-job/82421/2027-retirement-actuarial-graduate-trainee-consultant-programme</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t>BDO UK</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>2027 Associate Management Graduate Programme - London (Consulting)</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Deadline passed</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>https://targetjobs.co.uk/jobs/2027-associate-management-graduate-programme-london-245547</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
           <t>Kubrick Group</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>Data &amp; AI Consultant (register interest, Sep 2026+ cohorts)</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr"/>
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>Excludes Computer Science degree holders</t>
         </is>
       </c>
-      <c r="E28" s="5" t="inlineStr">
+      <c r="E29" s="5" t="inlineStr">
         <is>
           <t>https://targetjobs.co.uk/jobs/data-ai-consultant-register-your-interest-237573</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E28"/>
+  <autoFilter ref="A1:E29"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
@@ -8077,6 +8599,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -13669,19 +14192,27 @@
       </c>
       <c r="D147" s="2" t="inlineStr">
         <is>
-          <t>NOT YET CHECKED</t>
+          <t>Roles found</t>
         </is>
       </c>
       <c r="E147" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F147" s="2" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="F147" s="2" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
       <c r="G147" s="5" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/razorpaysoftwareprivatelimited</t>
-        </is>
-      </c>
-      <c r="H147" s="2" t="inlineStr"/>
+          <t>https://razorpay.com/jobs/</t>
+        </is>
+      </c>
+      <c r="H147" s="2" t="inlineStr">
+        <is>
+          <t>Junior Analyst – Business Operations (TCV, Sep 2025) likely closed. Listings are from fresher aggregators — confirm on razorpay.com/jobs.</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="n">
@@ -13699,19 +14230,27 @@
       </c>
       <c r="D148" s="2" t="inlineStr">
         <is>
-          <t>NOT YET CHECKED</t>
+          <t>No suitable role open</t>
         </is>
       </c>
       <c r="E148" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="F148" s="2" t="inlineStr"/>
+      <c r="F148" s="2" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
       <c r="G148" s="5" t="inlineStr">
         <is>
-          <t>https://www.icicicareers.com/</t>
-        </is>
-      </c>
-      <c r="H148" s="2" t="inlineStr"/>
+          <t>https://careers.idfcfirst.bank.in/in/en/campus</t>
+        </is>
+      </c>
+      <c r="H148" s="2" t="inlineStr">
+        <is>
+          <t>Fresher roles found are Relationship Manager / Assistant Manager / Customer Service (ICICI ₹3.1 LPA, HDFC ₹4.5 LPA, Axis ₹4.6 LPA) — sales/service, excluded. IDFC FIRST Management Trainee is a campus (MBA) route. Yes Bank Trainee (credit analysis) is Indore only.</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="n">
@@ -13729,19 +14268,27 @@
       </c>
       <c r="D149" s="2" t="inlineStr">
         <is>
-          <t>NOT YET CHECKED</t>
+          <t>No suitable role open</t>
         </is>
       </c>
       <c r="E149" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="F149" s="2" t="inlineStr"/>
+      <c r="F149" s="2" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
       <c r="G149" s="5" t="inlineStr">
         <is>
           <t>https://sbi.co.in/web/careers</t>
         </is>
       </c>
-      <c r="H149" s="2" t="inlineStr"/>
+      <c r="H149" s="2" t="inlineStr">
+        <is>
+          <t>SBI PO 2026 (1,500 posts) closed 8 Jul 2026; SCO notices closed Mar 2026. No data-analyst notification open.</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="n">
@@ -13759,19 +14306,27 @@
       </c>
       <c r="D150" s="2" t="inlineStr">
         <is>
-          <t>NOT YET CHECKED</t>
+          <t>Roles found</t>
         </is>
       </c>
       <c r="E150" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F150" s="2" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="F150" s="2" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
       <c r="G150" s="5" t="inlineStr">
         <is>
           <t>https://www.google.com/about/careers/applications/jobs/results/?location=India</t>
         </is>
       </c>
-      <c r="H150" s="2" t="inlineStr"/>
+      <c r="H150" s="2" t="inlineStr">
+        <is>
+          <t>Google Business Analyst (gTech; Planning &amp; Analytics) appear only as past listings. No India results for Microsoft, Salesforce, SAP, Adobe, Cisco, LinkedIn, ServiceNow, Snowflake, Databricks in one combined search — coverage of this group is partial.</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="n">
@@ -13789,19 +14344,27 @@
       </c>
       <c r="D151" s="2" t="inlineStr">
         <is>
-          <t>NOT YET CHECKED</t>
+          <t>Roles found</t>
         </is>
       </c>
       <c r="E151" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F151" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F151" s="2" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
       <c r="G151" s="5" t="inlineStr">
         <is>
           <t>https://www.freshworks.com/company/careers/</t>
         </is>
       </c>
-      <c r="H151" s="2" t="inlineStr"/>
+      <c r="H151" s="2" t="inlineStr">
+        <is>
+          <t>Freshworks BA – Revenue Operations (Chennai) expired. Delhivery listed with ~38 data-analyst openings (Naukri, May 2026) — no specific posting found. No results for Zoho, Postman, Chargebee, InMobi, Navi, Angel One; PolicyBazaar campus role is Relationship Manager.</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="n">
@@ -17744,7 +18307,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>195</v>
+        <v>200</v>
       </c>
     </row>
     <row r="4">
@@ -17754,7 +18317,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>58</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5">
@@ -17774,7 +18337,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7">
@@ -17943,7 +18506,7 @@
       <c r="A24" s="2" t="inlineStr"/>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>DEADLINES: a date is only recorded when a search result states it explicitly. Anything else is 'Rolling'. Deadline Source names the site the date came from (company site, Gradcracker, Bright Network, TargetJobs, Prospects, etc.).</t>
+          <t>SEARCH LIMIT: the session allows 200 web searches per turn. That limit was reached after UK rows 1–145, all 50 added UK companies and India rows 146–150. The remaining India companies (India rows 151–179 and added India rows 230–259) show 'NOT YET CHECKED' in Coverage; send 'continue' to resume from progress.jsonl.</t>
         </is>
       </c>
     </row>
@@ -17951,7 +18514,7 @@
       <c r="A25" s="2" t="inlineStr"/>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>SALARY / START / REQUIREMENTS: recorded only when the search result states them; otherwise 'Not stated'.</t>
+          <t>GROUPED INDIA ROWS 149 and 150 were covered by combined searches, so several companies inside those groups were not individually checked (listed under CHECK MANUALLY).</t>
         </is>
       </c>
     </row>
@@ -17959,7 +18522,7 @@
       <c r="A26" s="2" t="inlineStr"/>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>FIT SCORE: computed by score.py from the role family, seniority, skills mentioned, location and domain, per Section 5. Roles under 55 are moved to 'Closed - Excluded'.</t>
+          <t>DEADLINES: a date is only recorded when a search result states it explicitly. Anything else is 'Rolling'. Deadline Source names the site the date came from (company site, Gradcracker, Bright Network, TargetJobs, Prospects, etc.).</t>
         </is>
       </c>
     </row>
@@ -17967,7 +18530,7 @@
       <c r="A27" s="2" t="inlineStr"/>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>GROUPED ENTRIES (e.g. 'India private banks', 'India big-tech arms', 'India SaaS'): treated as one Coverage row each; up to 3 best roles across the whole group are listed, with the actual employer named in the Role Title.</t>
+          <t>SALARY / START / REQUIREMENTS: recorded only when the search result states them; otherwise 'Not stated'.</t>
         </is>
       </c>
     </row>
@@ -17975,7 +18538,7 @@
       <c r="A28" s="2" t="inlineStr"/>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Companies that also appear in both lists (e.g. Razorpay, PhonePe, ICICI/HDFC/Axis/Kotak in the UK list) were searched for openings in the region of the row: UK rows look for UK roles; India rows look for India roles. Indian banks and Gulf banks listed under 'UK' have no UK graduate hiring found unless stated.</t>
+          <t>FIT SCORE: computed by score.py from the role family, seniority, skills mentioned, location and domain, per Section 5. Roles under 55 are moved to 'Closed - Excluded'.</t>
         </is>
       </c>
     </row>
@@ -17983,7 +18546,7 @@
       <c r="A29" s="2" t="inlineStr"/>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Sheet 'Closed / Excluded' is named 'Closed - Excluded' because Excel forbids '/' in sheet names.</t>
+          <t>GROUPED ENTRIES (e.g. 'India private banks', 'India big-tech arms', 'India SaaS'): treated as one Coverage row each; up to 3 best roles across the whole group are listed, with the actual employer named in the Role Title.</t>
         </is>
       </c>
     </row>
@@ -17991,107 +18554,107 @@
       <c r="A30" s="2" t="inlineStr"/>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Checkpointing: results are appended to progress.jsonl per company and the workbook is rebuilt after each batch of companies.</t>
+          <t>Companies that also appear in both lists (e.g. Razorpay, PhonePe, ICICI/HDFC/Axis/Kotak in the UK list) were searched for openings in the region of the row: UK rows look for UK roles; India rows look for India roles. Indian banks and Gulf banks listed under 'UK' have no UK graduate hiring found unless stated.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr"/>
-      <c r="B31" s="2" t="inlineStr"/>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Sheet 'Closed / Excluded' is named 'Closed - Excluded' because Excel forbids '/' in sheet names.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="13" t="inlineStr">
+      <c r="A32" s="2" t="inlineStr"/>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Checkpointing: results are appended to progress.jsonl per company and the workbook is rebuilt after each batch of companies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr"/>
+      <c r="B33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="13" t="inlineStr">
         <is>
           <t>ALREADY-APPLIED: LIVE DEADLINES</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>Same role you applied for — confirm your application covers this cycle</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>Bain &amp; Company: Associate Consultant 2027 (London) — 23:59 BST — https://www.brightnetwork.co.uk/graduate-jobs/bain-company/associate-consultant-2027</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>Roland Berger: Junior Consultant 2027 (London) — cover letter required — https://www.rolandberger.com/en/Join/All-Jobs/Junior-Consultant-2027-REF4503I.html</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Kearney: Business Analyst 2027 (London) — rolling screening — https://www.iagora.com/work/en/offer/graduate-programme-united-kingdom-finance/6303561</t>
+          <t>Bain &amp; Company: Associate Consultant 2027 (London) — 23:59 BST — https://www.brightnetwork.co.uk/graduate-jobs/bain-company/associate-consultant-2027</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Roland Berger: Junior Consultant 2027 (London) — cover letter required — https://www.rolandberger.com/en/Join/All-Jobs/Junior-Consultant-2027-REF4503I.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Kearney: Business Analyst 2027 (London) — rolling screening — https://www.iagora.com/work/en/offer/graduate-programme-united-kingdom-finance/6303561</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
           <t>Rolling</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>Boston Consulting Group (BCG): Graduate Associate (London) — last cycle closed 23 Oct; 2026 date unconfirmed — https://careers.bcg.com/global/en/locations/united-kingdom/associate-jobs</t>
         </is>
       </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr"/>
-      <c r="B37" s="2" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="13" t="inlineStr">
-        <is>
-          <t>CHECK MANUALLY</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr"/>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>PwC (UK) (UK) — Check PwC UK Technology &amp; Data graduate 2027 listings directly</t>
-        </is>
-      </c>
+      <c r="B39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr"/>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>American Express (UK) — Amex UK 2027 graduate analyst schemes (Brighton) — not found by search; past cycles closed ~10 Nov</t>
-        </is>
-      </c>
+      <c r="A40" s="13" t="inlineStr">
+        <is>
+          <t>CHECK MANUALLY</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr"/>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Bloomberg (UK) — Bloomberg London grad Financial Data Analyst / Analytics &amp; Sales 2027 — not indexed by search</t>
+          <t>PwC (UK) (UK) — Check PwC UK Technology &amp; Data graduate 2027 listings directly</t>
         </is>
       </c>
     </row>
@@ -18099,7 +18662,7 @@
       <c r="A42" s="2" t="inlineStr"/>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>L.E.K. Consulting (UK) — L.E.K. London Associate 2027 — check regional vacancy page</t>
+          <t>American Express (UK) — Amex UK 2027 graduate analyst schemes (Brighton) — not found by search; past cycles closed ~10 Nov</t>
         </is>
       </c>
     </row>
@@ -18107,7 +18670,7 @@
       <c r="A43" s="2" t="inlineStr"/>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>abrdn (Aberdeen Group) (UK) — abrdn/Aberdeen 2027 graduate programme — last cycle closed ~18 Oct; not found by search</t>
+          <t>Bloomberg (UK) — Bloomberg London grad Financial Data Analyst / Analytics &amp; Sales 2027 — not indexed by search</t>
         </is>
       </c>
     </row>
@@ -18115,7 +18678,7 @@
       <c r="A44" s="2" t="inlineStr"/>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Man Group (UK) — Man Group Solutions Graduate Analyst — check Greenhouse board for intake year/deadline</t>
+          <t>L.E.K. Consulting (UK) — L.E.K. London Associate 2027 — check regional vacancy page</t>
         </is>
       </c>
     </row>
@@ -18123,7 +18686,7 @@
       <c r="A45" s="2" t="inlineStr"/>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Google (UK) — Google UK — careers site not indexed; check jobs search for 'graduate' / 'associate' in London</t>
+          <t>abrdn (Aberdeen Group) (UK) — abrdn/Aberdeen 2027 graduate programme — last cycle closed ~18 Oct; not found by search</t>
         </is>
       </c>
     </row>
@@ -18131,7 +18694,7 @@
       <c r="A46" s="2" t="inlineStr"/>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Santander (UK) (UK) — Santander UK — confirm whether any direct-entry 2027 graduate role exists (tracker says Nov 2026 close)</t>
+          <t>Man Group (UK) — Man Group Solutions Graduate Analyst — check Greenhouse board for intake year/deadline</t>
         </is>
       </c>
     </row>
@@ -18139,7 +18702,7 @@
       <c r="A47" s="2" t="inlineStr"/>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>BNP Paribas (UK) (UK) — BNP Paribas London 2027 Technology Graduate — check whether a business-analysis stream exists</t>
+          <t>Google (UK) — Google UK — careers site not indexed; check jobs search for 'graduate' / 'associate' in London</t>
         </is>
       </c>
     </row>
@@ -18147,7 +18710,7 @@
       <c r="A48" s="2" t="inlineStr"/>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>FactSet (UK) — FactSet London Client Solutions Associate — confirm if you'd consider a client-facing analyst role</t>
+          <t>Santander (UK) (UK) — Santander UK — confirm whether any direct-entry 2027 graduate role exists (tracker says Nov 2026 close)</t>
         </is>
       </c>
     </row>
@@ -18155,7 +18718,7 @@
       <c r="A49" s="2" t="inlineStr"/>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>PA Consulting (UK) — PA Consulting 2027 graduate — not indexed; last cycle closed 7 Nov</t>
+          <t>BNP Paribas (UK) (UK) — BNP Paribas London 2027 Technology Graduate — check whether a business-analysis stream exists</t>
         </is>
       </c>
     </row>
@@ -18163,7 +18726,7 @@
       <c r="A50" s="2" t="inlineStr"/>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Slalom (UK) — Slalom London — careers site not indexed</t>
+          <t>FactSet (UK) — FactSet London Client Solutions Associate — confirm if you'd consider a client-facing analyst role</t>
         </is>
       </c>
     </row>
@@ -18171,7 +18734,7 @@
       <c r="A51" s="2" t="inlineStr"/>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Kainos (UK) — Kainos graduate Business Analyst 2027 — search returned no results; check kainos.com/careers/early-careers</t>
+          <t>PA Consulting (UK) — PA Consulting 2027 graduate — not indexed; last cycle closed 7 Nov</t>
         </is>
       </c>
     </row>
@@ -18179,7 +18742,7 @@
       <c r="A52" s="2" t="inlineStr"/>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Grant Thornton (UK) (UK) — Grant Thornton UK 2027 Consulting / Risk graduate — not indexed</t>
+          <t>Slalom (UK) — Slalom London — careers site not indexed</t>
         </is>
       </c>
     </row>
@@ -18187,7 +18750,7 @@
       <c r="A53" s="2" t="inlineStr"/>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Zanders (UK) — Zanders UK graduate consultant — check graduate recruitment page for a London opening</t>
+          <t>Kainos (UK) — Kainos graduate Business Analyst 2027 — search returned no results; check kainos.com/careers/early-careers</t>
         </is>
       </c>
     </row>
@@ -18195,7 +18758,7 @@
       <c r="A54" s="2" t="inlineStr"/>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Plaid (UK) — Plaid London — careers site not indexed</t>
+          <t>Grant Thornton (UK) (UK) — Grant Thornton UK 2027 Consulting / Risk graduate — not indexed</t>
         </is>
       </c>
     </row>
@@ -18203,7 +18766,7 @@
       <c r="A55" s="2" t="inlineStr"/>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Cisco (UK) (UK) — Cisco UK early careers (Feltham) — check jobs.cisco.com for 2027 graduate analyst roles</t>
+          <t>Zanders (UK) — Zanders UK graduate consultant — check graduate recruitment page for a London opening</t>
         </is>
       </c>
     </row>
@@ -18211,7 +18774,7 @@
       <c r="A56" s="2" t="inlineStr"/>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Spotify (UK) (UK) — Spotify London — check lifeatspotify for current Associate/Analyst early-career roles</t>
+          <t>Plaid (UK) — Plaid London — careers site not indexed</t>
         </is>
       </c>
     </row>
@@ -18219,7 +18782,7 @@
       <c r="A57" s="2" t="inlineStr"/>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn (UK) (UK) — LinkedIn Strategy &amp; Analytics pathway — check if a Dublin/London cohort is open</t>
+          <t>Cisco (UK) (UK) — Cisco UK early careers (Feltham) — check jobs.cisco.com for 2027 graduate analyst roles</t>
         </is>
       </c>
     </row>
@@ -18227,7 +18790,7 @@
       <c r="A58" s="2" t="inlineStr"/>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Palantir (UK) (UK) — Palantir London Deployment Strategist (new grad) — check palantir.com/careers</t>
+          <t>Spotify (UK) (UK) — Spotify London — check lifeatspotify for current Associate/Analyst early-career roles</t>
         </is>
       </c>
     </row>
@@ -18235,7 +18798,7 @@
       <c r="A59" s="2" t="inlineStr"/>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Mercer (Marsh McLennan) (UK) — Mercer UK 2027 graduate (actuarial/wealth/consulting analyst) — not indexed; check careers.marshmclennan.com</t>
+          <t>LinkedIn (UK) (UK) — LinkedIn Strategy &amp; Analytics pathway — check if a Dublin/London cohort is open</t>
         </is>
       </c>
     </row>
@@ -18243,7 +18806,7 @@
       <c r="A60" s="2" t="inlineStr"/>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Berkeley Research Group (BRG) (UK) — BRG London Associate (2027) — check thinkbrg.com careers</t>
+          <t>Palantir (UK) (UK) — Palantir London Deployment Strategist (new grad) — check palantir.com/careers</t>
         </is>
       </c>
     </row>
@@ -18251,7 +18814,7 @@
       <c r="A61" s="2" t="inlineStr"/>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Razorpay (India) — not yet checked</t>
+          <t>Mercer (Marsh McLennan) (UK) — Mercer UK 2027 graduate (actuarial/wealth/consulting analyst) — not indexed; check careers.marshmclennan.com</t>
         </is>
       </c>
     </row>
@@ -18259,7 +18822,7 @@
       <c r="A62" s="2" t="inlineStr"/>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>India private banks (ICICI, HDFC, Axis, Kotak, IDFC First, Yes) (India) — not yet checked</t>
+          <t>Berkeley Research Group (BRG) (UK) — BRG London Associate (2027) — check thinkbrg.com careers</t>
         </is>
       </c>
     </row>
@@ -18267,7 +18830,7 @@
       <c r="A63" s="2" t="inlineStr"/>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>SBI (State Bank of India) (India) — not yet checked</t>
+          <t>India private banks (ICICI, HDFC, Axis, Kotak, IDFC First, Yes) (India) — Kotak / HDFC / ICICI analytics or credit-analyst fresher roles — check each bank's careers portal</t>
         </is>
       </c>
     </row>
@@ -18275,7 +18838,7 @@
       <c r="A64" s="2" t="inlineStr"/>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>India big-tech arms (Google, Microsoft, Amazon [done], Salesforce, Oracle, SAP, Adobe, Cisco, Uber, LinkedIn, ServiceNow, Snowflake, Databricks) (India) — not yet checked</t>
+          <t>India big-tech arms (Google, Microsoft, Amazon [done], Salesforce, Oracle, SAP, Adobe, Cisco, Uber, LinkedIn, ServiceNow, Snowflake, Databricks) (India) — India big-tech group: Microsoft, Salesforce, SAP, Adobe, Cisco, LinkedIn, ServiceNow, Snowflake, Databricks not individually searched</t>
         </is>
       </c>
     </row>
@@ -18283,7 +18846,7 @@
       <c r="A65" s="2" t="inlineStr"/>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>India SaaS (Freshworks, Zoho, Postman, Chargebee, BrowserStack, InMobi, Delhivery, PolicyBazaar, Navi, Angel One) (India) — not yet checked</t>
+          <t>India SaaS (Freshworks, Zoho, Postman, Chargebee, BrowserStack, InMobi, Delhivery, PolicyBazaar, Navi, Angel One) (India) — India SaaS group: Zoho, Postman, Chargebee, InMobi, Navi, Angel One, Delhivery — search careers pages individually</t>
         </is>
       </c>
     </row>

</xml_diff>